<commit_message>
small update in megatrends_RF.xlsx
</commit_message>
<xml_diff>
--- a/progress/megatrends_RF.xlsx
+++ b/progress/megatrends_RF.xlsx
@@ -565,7 +565,22 @@
     <t xml:space="preserve">Road density</t>
   </si>
   <si>
-    <t xml:space="preserve">length of road network per area</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">length of road network per area
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color indexed="2"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">which kind of road?</t>
+    </r>
   </si>
   <si>
     <t>BD_TOPO</t>
@@ -6030,7 +6045,7 @@
       <c r="JM14" s="25"/>
       <c r="JN14" s="25"/>
     </row>
-    <row r="15" s="14" customFormat="1" ht="51">
+    <row r="15" s="14" customFormat="1" ht="25.5">
       <c r="A15" s="26" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
add the PCA based on WS4 group discussion
</commit_message>
<xml_diff>
--- a/progress/megatrends_RF.xlsx
+++ b/progress/megatrends_RF.xlsx
@@ -550,10 +550,12 @@
     <t xml:space="preserve">INSEE - ADMIN_EXPRESS</t>
   </si>
   <si>
-    <t>Pop_dens</t>
-  </si>
-  <si>
-    <t>https://www.insee.fr/fr/statistiques/3698339</t>
+    <t xml:space="preserve">Pop_dens - commune
+JRC - 100m raster?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.insee.fr/fr/statistiques/3698339
+https://www.insee.fr/fr/statistiques/8272002</t>
   </si>
   <si>
     <t xml:space="preserve">1876 - 2022</t>
@@ -1071,7 +1073,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1181,6 +1183,9 @@
     </xf>
     <xf fontId="0" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="6" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1801,7 +1806,7 @@
     <col customWidth="1" min="5" max="5" width="58.8515625"/>
     <col customWidth="1" min="6" max="6" width="32.140625"/>
     <col customWidth="1" min="7" max="7" width="31.140625"/>
-    <col customWidth="1" min="9" max="9" style="2" width="32.00390625"/>
+    <col customWidth="1" min="9" max="9" style="2" width="36.140625"/>
     <col customWidth="1" min="10" max="10" width="32.28125"/>
     <col customWidth="1" min="11" max="11" width="24.00390625"/>
     <col customWidth="1" min="12" max="12" width="12.140625"/>
@@ -7287,7 +7292,7 @@
       <c r="JM19" s="10"/>
       <c r="JN19" s="10"/>
     </row>
-    <row r="20" s="39" customFormat="1" ht="42.75">
+    <row r="20" s="39" customFormat="1" ht="51">
       <c r="A20" s="27" t="s">
         <v>132</v>
       </c>
@@ -7310,10 +7315,10 @@
         <v>162</v>
       </c>
       <c r="H20" s="27"/>
-      <c r="I20" s="32" t="s">
+      <c r="I20" s="40" t="s">
         <v>163</v>
       </c>
-      <c r="J20" s="40"/>
+      <c r="J20" s="41"/>
       <c r="K20" s="27" t="s">
         <v>164</v>
       </c>
@@ -7324,268 +7329,268 @@
       <c r="N20" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="O20" s="41"/>
-      <c r="P20" s="41"/>
-      <c r="Q20" s="41"/>
-      <c r="R20" s="41"/>
-      <c r="S20" s="41"/>
-      <c r="T20" s="41"/>
-      <c r="U20" s="41"/>
-      <c r="V20" s="41"/>
-      <c r="W20" s="41"/>
-      <c r="X20" s="41"/>
-      <c r="Y20" s="41"/>
-      <c r="Z20" s="41"/>
-      <c r="AA20" s="41"/>
-      <c r="AB20" s="41"/>
-      <c r="AC20" s="41"/>
-      <c r="AD20" s="41"/>
-      <c r="AE20" s="41"/>
-      <c r="AF20" s="41"/>
-      <c r="AG20" s="41"/>
-      <c r="AH20" s="41"/>
-      <c r="AI20" s="41"/>
-      <c r="AJ20" s="41"/>
-      <c r="AK20" s="41"/>
-      <c r="AL20" s="41"/>
-      <c r="AM20" s="41"/>
-      <c r="AN20" s="41"/>
-      <c r="AO20" s="41"/>
-      <c r="AP20" s="41"/>
-      <c r="AQ20" s="41"/>
-      <c r="AR20" s="41"/>
-      <c r="AS20" s="41"/>
-      <c r="AT20" s="41"/>
-      <c r="AU20" s="41"/>
-      <c r="AV20" s="41"/>
-      <c r="AW20" s="41"/>
-      <c r="AX20" s="41"/>
-      <c r="AY20" s="41"/>
-      <c r="AZ20" s="41"/>
-      <c r="BA20" s="41"/>
-      <c r="BB20" s="41"/>
-      <c r="BC20" s="41"/>
-      <c r="BD20" s="41"/>
-      <c r="BE20" s="41"/>
-      <c r="BF20" s="41"/>
-      <c r="BG20" s="41"/>
-      <c r="BH20" s="41"/>
-      <c r="BI20" s="41"/>
-      <c r="BJ20" s="41"/>
-      <c r="BK20" s="41"/>
-      <c r="BL20" s="41"/>
-      <c r="BM20" s="41"/>
-      <c r="BN20" s="41"/>
-      <c r="BO20" s="41"/>
-      <c r="BP20" s="41"/>
-      <c r="BQ20" s="41"/>
-      <c r="BR20" s="41"/>
-      <c r="BS20" s="41"/>
-      <c r="BT20" s="41"/>
-      <c r="BU20" s="41"/>
-      <c r="BV20" s="41"/>
-      <c r="BW20" s="41"/>
-      <c r="BX20" s="41"/>
-      <c r="BY20" s="41"/>
-      <c r="BZ20" s="41"/>
-      <c r="CA20" s="41"/>
-      <c r="CB20" s="41"/>
-      <c r="CC20" s="41"/>
-      <c r="CD20" s="41"/>
-      <c r="CE20" s="41"/>
-      <c r="CF20" s="41"/>
-      <c r="CG20" s="41"/>
-      <c r="CH20" s="41"/>
-      <c r="CI20" s="41"/>
-      <c r="CJ20" s="41"/>
-      <c r="CK20" s="41"/>
-      <c r="CL20" s="41"/>
-      <c r="CM20" s="41"/>
-      <c r="CN20" s="41"/>
-      <c r="CO20" s="41"/>
-      <c r="CP20" s="41"/>
-      <c r="CQ20" s="41"/>
-      <c r="CR20" s="41"/>
-      <c r="CS20" s="41"/>
-      <c r="CT20" s="41"/>
-      <c r="CU20" s="41"/>
-      <c r="CV20" s="41"/>
-      <c r="CW20" s="41"/>
-      <c r="CX20" s="41"/>
-      <c r="CY20" s="41"/>
-      <c r="CZ20" s="41"/>
-      <c r="DA20" s="41"/>
-      <c r="DB20" s="41"/>
-      <c r="DC20" s="41"/>
-      <c r="DD20" s="41"/>
-      <c r="DE20" s="41"/>
-      <c r="DF20" s="41"/>
-      <c r="DG20" s="41"/>
-      <c r="DH20" s="41"/>
-      <c r="DI20" s="41"/>
-      <c r="DJ20" s="41"/>
-      <c r="DK20" s="41"/>
-      <c r="DL20" s="41"/>
-      <c r="DM20" s="41"/>
-      <c r="DN20" s="41"/>
-      <c r="DO20" s="41"/>
-      <c r="DP20" s="41"/>
-      <c r="DQ20" s="41"/>
-      <c r="DR20" s="41"/>
-      <c r="DS20" s="41"/>
-      <c r="DT20" s="41"/>
-      <c r="DU20" s="41"/>
-      <c r="DV20" s="41"/>
-      <c r="DW20" s="41"/>
-      <c r="DX20" s="41"/>
-      <c r="DY20" s="41"/>
-      <c r="DZ20" s="41"/>
-      <c r="EA20" s="41"/>
-      <c r="EB20" s="41"/>
-      <c r="EC20" s="41"/>
-      <c r="ED20" s="41"/>
-      <c r="EE20" s="41"/>
-      <c r="EF20" s="41"/>
-      <c r="EG20" s="41"/>
-      <c r="EH20" s="41"/>
-      <c r="EI20" s="41"/>
-      <c r="EJ20" s="41"/>
-      <c r="EK20" s="41"/>
-      <c r="EL20" s="41"/>
-      <c r="EM20" s="41"/>
-      <c r="EN20" s="41"/>
-      <c r="EO20" s="41"/>
-      <c r="EP20" s="41"/>
-      <c r="EQ20" s="41"/>
-      <c r="ER20" s="41"/>
-      <c r="ES20" s="41"/>
-      <c r="ET20" s="41"/>
-      <c r="EU20" s="41"/>
-      <c r="EV20" s="41"/>
-      <c r="EW20" s="41"/>
-      <c r="EX20" s="41"/>
-      <c r="EY20" s="41"/>
-      <c r="EZ20" s="41"/>
-      <c r="FA20" s="41"/>
-      <c r="FB20" s="41"/>
-      <c r="FC20" s="41"/>
-      <c r="FD20" s="41"/>
-      <c r="FE20" s="41"/>
-      <c r="FF20" s="41"/>
-      <c r="FG20" s="41"/>
-      <c r="FH20" s="41"/>
-      <c r="FI20" s="41"/>
-      <c r="FJ20" s="41"/>
-      <c r="FK20" s="41"/>
-      <c r="FL20" s="41"/>
-      <c r="FM20" s="41"/>
-      <c r="FN20" s="41"/>
-      <c r="FO20" s="41"/>
-      <c r="FP20" s="41"/>
-      <c r="FQ20" s="41"/>
-      <c r="FR20" s="41"/>
-      <c r="FS20" s="41"/>
-      <c r="FT20" s="41"/>
-      <c r="FU20" s="41"/>
-      <c r="FV20" s="41"/>
-      <c r="FW20" s="41"/>
-      <c r="FX20" s="41"/>
-      <c r="FY20" s="41"/>
-      <c r="FZ20" s="41"/>
-      <c r="GA20" s="41"/>
-      <c r="GB20" s="41"/>
-      <c r="GC20" s="41"/>
-      <c r="GD20" s="41"/>
-      <c r="GE20" s="41"/>
-      <c r="GF20" s="41"/>
-      <c r="GG20" s="41"/>
-      <c r="GH20" s="41"/>
-      <c r="GI20" s="41"/>
-      <c r="GJ20" s="41"/>
-      <c r="GK20" s="41"/>
-      <c r="GL20" s="41"/>
-      <c r="GM20" s="41"/>
-      <c r="GN20" s="41"/>
-      <c r="GO20" s="41"/>
-      <c r="GP20" s="41"/>
-      <c r="GQ20" s="41"/>
-      <c r="GR20" s="41"/>
-      <c r="GS20" s="41"/>
-      <c r="GT20" s="41"/>
-      <c r="GU20" s="41"/>
-      <c r="GV20" s="41"/>
-      <c r="GW20" s="41"/>
-      <c r="GX20" s="41"/>
-      <c r="GY20" s="41"/>
-      <c r="GZ20" s="41"/>
-      <c r="HA20" s="41"/>
-      <c r="HB20" s="41"/>
-      <c r="HC20" s="41"/>
-      <c r="HD20" s="41"/>
-      <c r="HE20" s="41"/>
-      <c r="HF20" s="41"/>
-      <c r="HG20" s="41"/>
-      <c r="HH20" s="41"/>
-      <c r="HI20" s="41"/>
-      <c r="HJ20" s="41"/>
-      <c r="HK20" s="41"/>
-      <c r="HL20" s="41"/>
-      <c r="HM20" s="41"/>
-      <c r="HN20" s="41"/>
-      <c r="HO20" s="41"/>
-      <c r="HP20" s="41"/>
-      <c r="HQ20" s="41"/>
-      <c r="HR20" s="41"/>
-      <c r="HS20" s="41"/>
-      <c r="HT20" s="41"/>
-      <c r="HU20" s="41"/>
-      <c r="HV20" s="41"/>
-      <c r="HW20" s="41"/>
-      <c r="HX20" s="41"/>
-      <c r="HY20" s="41"/>
-      <c r="HZ20" s="41"/>
-      <c r="IA20" s="41"/>
-      <c r="IB20" s="41"/>
-      <c r="IC20" s="41"/>
-      <c r="ID20" s="41"/>
-      <c r="IE20" s="41"/>
-      <c r="IF20" s="41"/>
-      <c r="IG20" s="41"/>
-      <c r="IH20" s="41"/>
-      <c r="II20" s="41"/>
-      <c r="IJ20" s="41"/>
-      <c r="IK20" s="41"/>
-      <c r="IL20" s="41"/>
-      <c r="IM20" s="41"/>
-      <c r="IN20" s="41"/>
-      <c r="IO20" s="41"/>
-      <c r="IP20" s="41"/>
-      <c r="IQ20" s="41"/>
-      <c r="IR20" s="41"/>
-      <c r="IS20" s="41"/>
-      <c r="IT20" s="41"/>
-      <c r="IU20" s="41"/>
-      <c r="IV20" s="41"/>
-      <c r="IW20" s="41"/>
-      <c r="IX20" s="41"/>
-      <c r="IY20" s="41"/>
-      <c r="IZ20" s="41"/>
-      <c r="JA20" s="41"/>
-      <c r="JB20" s="41"/>
-      <c r="JC20" s="41"/>
-      <c r="JD20" s="41"/>
-      <c r="JE20" s="41"/>
-      <c r="JF20" s="41"/>
-      <c r="JG20" s="41"/>
-      <c r="JH20" s="41"/>
-      <c r="JI20" s="41"/>
-      <c r="JJ20" s="41"/>
-      <c r="JK20" s="41"/>
-      <c r="JL20" s="41"/>
-      <c r="JM20" s="41"/>
-      <c r="JN20" s="41"/>
+      <c r="O20" s="42"/>
+      <c r="P20" s="42"/>
+      <c r="Q20" s="42"/>
+      <c r="R20" s="42"/>
+      <c r="S20" s="42"/>
+      <c r="T20" s="42"/>
+      <c r="U20" s="42"/>
+      <c r="V20" s="42"/>
+      <c r="W20" s="42"/>
+      <c r="X20" s="42"/>
+      <c r="Y20" s="42"/>
+      <c r="Z20" s="42"/>
+      <c r="AA20" s="42"/>
+      <c r="AB20" s="42"/>
+      <c r="AC20" s="42"/>
+      <c r="AD20" s="42"/>
+      <c r="AE20" s="42"/>
+      <c r="AF20" s="42"/>
+      <c r="AG20" s="42"/>
+      <c r="AH20" s="42"/>
+      <c r="AI20" s="42"/>
+      <c r="AJ20" s="42"/>
+      <c r="AK20" s="42"/>
+      <c r="AL20" s="42"/>
+      <c r="AM20" s="42"/>
+      <c r="AN20" s="42"/>
+      <c r="AO20" s="42"/>
+      <c r="AP20" s="42"/>
+      <c r="AQ20" s="42"/>
+      <c r="AR20" s="42"/>
+      <c r="AS20" s="42"/>
+      <c r="AT20" s="42"/>
+      <c r="AU20" s="42"/>
+      <c r="AV20" s="42"/>
+      <c r="AW20" s="42"/>
+      <c r="AX20" s="42"/>
+      <c r="AY20" s="42"/>
+      <c r="AZ20" s="42"/>
+      <c r="BA20" s="42"/>
+      <c r="BB20" s="42"/>
+      <c r="BC20" s="42"/>
+      <c r="BD20" s="42"/>
+      <c r="BE20" s="42"/>
+      <c r="BF20" s="42"/>
+      <c r="BG20" s="42"/>
+      <c r="BH20" s="42"/>
+      <c r="BI20" s="42"/>
+      <c r="BJ20" s="42"/>
+      <c r="BK20" s="42"/>
+      <c r="BL20" s="42"/>
+      <c r="BM20" s="42"/>
+      <c r="BN20" s="42"/>
+      <c r="BO20" s="42"/>
+      <c r="BP20" s="42"/>
+      <c r="BQ20" s="42"/>
+      <c r="BR20" s="42"/>
+      <c r="BS20" s="42"/>
+      <c r="BT20" s="42"/>
+      <c r="BU20" s="42"/>
+      <c r="BV20" s="42"/>
+      <c r="BW20" s="42"/>
+      <c r="BX20" s="42"/>
+      <c r="BY20" s="42"/>
+      <c r="BZ20" s="42"/>
+      <c r="CA20" s="42"/>
+      <c r="CB20" s="42"/>
+      <c r="CC20" s="42"/>
+      <c r="CD20" s="42"/>
+      <c r="CE20" s="42"/>
+      <c r="CF20" s="42"/>
+      <c r="CG20" s="42"/>
+      <c r="CH20" s="42"/>
+      <c r="CI20" s="42"/>
+      <c r="CJ20" s="42"/>
+      <c r="CK20" s="42"/>
+      <c r="CL20" s="42"/>
+      <c r="CM20" s="42"/>
+      <c r="CN20" s="42"/>
+      <c r="CO20" s="42"/>
+      <c r="CP20" s="42"/>
+      <c r="CQ20" s="42"/>
+      <c r="CR20" s="42"/>
+      <c r="CS20" s="42"/>
+      <c r="CT20" s="42"/>
+      <c r="CU20" s="42"/>
+      <c r="CV20" s="42"/>
+      <c r="CW20" s="42"/>
+      <c r="CX20" s="42"/>
+      <c r="CY20" s="42"/>
+      <c r="CZ20" s="42"/>
+      <c r="DA20" s="42"/>
+      <c r="DB20" s="42"/>
+      <c r="DC20" s="42"/>
+      <c r="DD20" s="42"/>
+      <c r="DE20" s="42"/>
+      <c r="DF20" s="42"/>
+      <c r="DG20" s="42"/>
+      <c r="DH20" s="42"/>
+      <c r="DI20" s="42"/>
+      <c r="DJ20" s="42"/>
+      <c r="DK20" s="42"/>
+      <c r="DL20" s="42"/>
+      <c r="DM20" s="42"/>
+      <c r="DN20" s="42"/>
+      <c r="DO20" s="42"/>
+      <c r="DP20" s="42"/>
+      <c r="DQ20" s="42"/>
+      <c r="DR20" s="42"/>
+      <c r="DS20" s="42"/>
+      <c r="DT20" s="42"/>
+      <c r="DU20" s="42"/>
+      <c r="DV20" s="42"/>
+      <c r="DW20" s="42"/>
+      <c r="DX20" s="42"/>
+      <c r="DY20" s="42"/>
+      <c r="DZ20" s="42"/>
+      <c r="EA20" s="42"/>
+      <c r="EB20" s="42"/>
+      <c r="EC20" s="42"/>
+      <c r="ED20" s="42"/>
+      <c r="EE20" s="42"/>
+      <c r="EF20" s="42"/>
+      <c r="EG20" s="42"/>
+      <c r="EH20" s="42"/>
+      <c r="EI20" s="42"/>
+      <c r="EJ20" s="42"/>
+      <c r="EK20" s="42"/>
+      <c r="EL20" s="42"/>
+      <c r="EM20" s="42"/>
+      <c r="EN20" s="42"/>
+      <c r="EO20" s="42"/>
+      <c r="EP20" s="42"/>
+      <c r="EQ20" s="42"/>
+      <c r="ER20" s="42"/>
+      <c r="ES20" s="42"/>
+      <c r="ET20" s="42"/>
+      <c r="EU20" s="42"/>
+      <c r="EV20" s="42"/>
+      <c r="EW20" s="42"/>
+      <c r="EX20" s="42"/>
+      <c r="EY20" s="42"/>
+      <c r="EZ20" s="42"/>
+      <c r="FA20" s="42"/>
+      <c r="FB20" s="42"/>
+      <c r="FC20" s="42"/>
+      <c r="FD20" s="42"/>
+      <c r="FE20" s="42"/>
+      <c r="FF20" s="42"/>
+      <c r="FG20" s="42"/>
+      <c r="FH20" s="42"/>
+      <c r="FI20" s="42"/>
+      <c r="FJ20" s="42"/>
+      <c r="FK20" s="42"/>
+      <c r="FL20" s="42"/>
+      <c r="FM20" s="42"/>
+      <c r="FN20" s="42"/>
+      <c r="FO20" s="42"/>
+      <c r="FP20" s="42"/>
+      <c r="FQ20" s="42"/>
+      <c r="FR20" s="42"/>
+      <c r="FS20" s="42"/>
+      <c r="FT20" s="42"/>
+      <c r="FU20" s="42"/>
+      <c r="FV20" s="42"/>
+      <c r="FW20" s="42"/>
+      <c r="FX20" s="42"/>
+      <c r="FY20" s="42"/>
+      <c r="FZ20" s="42"/>
+      <c r="GA20" s="42"/>
+      <c r="GB20" s="42"/>
+      <c r="GC20" s="42"/>
+      <c r="GD20" s="42"/>
+      <c r="GE20" s="42"/>
+      <c r="GF20" s="42"/>
+      <c r="GG20" s="42"/>
+      <c r="GH20" s="42"/>
+      <c r="GI20" s="42"/>
+      <c r="GJ20" s="42"/>
+      <c r="GK20" s="42"/>
+      <c r="GL20" s="42"/>
+      <c r="GM20" s="42"/>
+      <c r="GN20" s="42"/>
+      <c r="GO20" s="42"/>
+      <c r="GP20" s="42"/>
+      <c r="GQ20" s="42"/>
+      <c r="GR20" s="42"/>
+      <c r="GS20" s="42"/>
+      <c r="GT20" s="42"/>
+      <c r="GU20" s="42"/>
+      <c r="GV20" s="42"/>
+      <c r="GW20" s="42"/>
+      <c r="GX20" s="42"/>
+      <c r="GY20" s="42"/>
+      <c r="GZ20" s="42"/>
+      <c r="HA20" s="42"/>
+      <c r="HB20" s="42"/>
+      <c r="HC20" s="42"/>
+      <c r="HD20" s="42"/>
+      <c r="HE20" s="42"/>
+      <c r="HF20" s="42"/>
+      <c r="HG20" s="42"/>
+      <c r="HH20" s="42"/>
+      <c r="HI20" s="42"/>
+      <c r="HJ20" s="42"/>
+      <c r="HK20" s="42"/>
+      <c r="HL20" s="42"/>
+      <c r="HM20" s="42"/>
+      <c r="HN20" s="42"/>
+      <c r="HO20" s="42"/>
+      <c r="HP20" s="42"/>
+      <c r="HQ20" s="42"/>
+      <c r="HR20" s="42"/>
+      <c r="HS20" s="42"/>
+      <c r="HT20" s="42"/>
+      <c r="HU20" s="42"/>
+      <c r="HV20" s="42"/>
+      <c r="HW20" s="42"/>
+      <c r="HX20" s="42"/>
+      <c r="HY20" s="42"/>
+      <c r="HZ20" s="42"/>
+      <c r="IA20" s="42"/>
+      <c r="IB20" s="42"/>
+      <c r="IC20" s="42"/>
+      <c r="ID20" s="42"/>
+      <c r="IE20" s="42"/>
+      <c r="IF20" s="42"/>
+      <c r="IG20" s="42"/>
+      <c r="IH20" s="42"/>
+      <c r="II20" s="42"/>
+      <c r="IJ20" s="42"/>
+      <c r="IK20" s="42"/>
+      <c r="IL20" s="42"/>
+      <c r="IM20" s="42"/>
+      <c r="IN20" s="42"/>
+      <c r="IO20" s="42"/>
+      <c r="IP20" s="42"/>
+      <c r="IQ20" s="42"/>
+      <c r="IR20" s="42"/>
+      <c r="IS20" s="42"/>
+      <c r="IT20" s="42"/>
+      <c r="IU20" s="42"/>
+      <c r="IV20" s="42"/>
+      <c r="IW20" s="42"/>
+      <c r="IX20" s="42"/>
+      <c r="IY20" s="42"/>
+      <c r="IZ20" s="42"/>
+      <c r="JA20" s="42"/>
+      <c r="JB20" s="42"/>
+      <c r="JC20" s="42"/>
+      <c r="JD20" s="42"/>
+      <c r="JE20" s="42"/>
+      <c r="JF20" s="42"/>
+      <c r="JG20" s="42"/>
+      <c r="JH20" s="42"/>
+      <c r="JI20" s="42"/>
+      <c r="JJ20" s="42"/>
+      <c r="JK20" s="42"/>
+      <c r="JL20" s="42"/>
+      <c r="JM20" s="42"/>
+      <c r="JN20" s="42"/>
     </row>
-    <row r="21" s="42" customFormat="1" ht="25.5">
+    <row r="21" s="43" customFormat="1" ht="25.5">
       <c r="A21" s="27" t="s">
         <v>132</v>
       </c>
@@ -7611,7 +7616,7 @@
       <c r="I21" s="32" t="s">
         <v>170</v>
       </c>
-      <c r="J21" s="40"/>
+      <c r="J21" s="41"/>
       <c r="K21" s="27">
         <v>2025</v>
       </c>
@@ -7620,971 +7625,971 @@
       </c>
       <c r="M21" s="27"/>
       <c r="N21" s="16"/>
-      <c r="O21" s="42"/>
-      <c r="P21" s="42"/>
-      <c r="Q21" s="42"/>
-      <c r="R21" s="42"/>
-      <c r="S21" s="42"/>
-      <c r="T21" s="42"/>
-      <c r="U21" s="42"/>
-      <c r="V21" s="42"/>
-      <c r="W21" s="42"/>
-      <c r="X21" s="42"/>
-      <c r="Y21" s="42"/>
-      <c r="Z21" s="42"/>
-      <c r="AA21" s="42"/>
-      <c r="AB21" s="42"/>
-      <c r="AC21" s="42"/>
-      <c r="AD21" s="42"/>
-      <c r="AE21" s="42"/>
-      <c r="AF21" s="42"/>
-      <c r="AG21" s="42"/>
-      <c r="AH21" s="42"/>
-      <c r="AI21" s="42"/>
-      <c r="AJ21" s="42"/>
-      <c r="AK21" s="42"/>
-      <c r="AL21" s="42"/>
-      <c r="AM21" s="42"/>
-      <c r="AN21" s="42"/>
-      <c r="AO21" s="42"/>
-      <c r="AP21" s="42"/>
-      <c r="AQ21" s="42"/>
-      <c r="AR21" s="42"/>
-      <c r="AS21" s="42"/>
-      <c r="AT21" s="42"/>
-      <c r="AU21" s="42"/>
-      <c r="AV21" s="42"/>
-      <c r="AW21" s="42"/>
-      <c r="AX21" s="42"/>
-      <c r="AY21" s="42"/>
-      <c r="AZ21" s="42"/>
-      <c r="BA21" s="42"/>
-      <c r="BB21" s="42"/>
-      <c r="BC21" s="42"/>
-      <c r="BD21" s="42"/>
-      <c r="BE21" s="42"/>
-      <c r="BF21" s="42"/>
-      <c r="BG21" s="42"/>
-      <c r="BH21" s="42"/>
-      <c r="BI21" s="42"/>
-      <c r="BJ21" s="42"/>
-      <c r="BK21" s="42"/>
-      <c r="BL21" s="42"/>
-      <c r="BM21" s="42"/>
-      <c r="BN21" s="42"/>
-      <c r="BO21" s="42"/>
-      <c r="BP21" s="42"/>
-      <c r="BQ21" s="42"/>
-      <c r="BR21" s="42"/>
-      <c r="BS21" s="42"/>
-      <c r="BT21" s="42"/>
-      <c r="BU21" s="42"/>
-      <c r="BV21" s="42"/>
-      <c r="BW21" s="42"/>
-      <c r="BX21" s="42"/>
-      <c r="BY21" s="42"/>
-      <c r="BZ21" s="42"/>
-      <c r="CA21" s="42"/>
-      <c r="CB21" s="42"/>
-      <c r="CC21" s="42"/>
-      <c r="CD21" s="42"/>
-      <c r="CE21" s="42"/>
-      <c r="CF21" s="42"/>
-      <c r="CG21" s="42"/>
-      <c r="CH21" s="42"/>
-      <c r="CI21" s="42"/>
-      <c r="CJ21" s="42"/>
-      <c r="CK21" s="42"/>
-      <c r="CL21" s="42"/>
-      <c r="CM21" s="42"/>
-      <c r="CN21" s="42"/>
-      <c r="CO21" s="42"/>
-      <c r="CP21" s="42"/>
-      <c r="CQ21" s="42"/>
-      <c r="CR21" s="42"/>
-      <c r="CS21" s="42"/>
-      <c r="CT21" s="42"/>
-      <c r="CU21" s="42"/>
-      <c r="CV21" s="42"/>
-      <c r="CW21" s="42"/>
-      <c r="CX21" s="42"/>
-      <c r="CY21" s="42"/>
-      <c r="CZ21" s="42"/>
-      <c r="DA21" s="42"/>
-      <c r="DB21" s="42"/>
-      <c r="DC21" s="42"/>
-      <c r="DD21" s="42"/>
-      <c r="DE21" s="42"/>
-      <c r="DF21" s="42"/>
-      <c r="DG21" s="42"/>
-      <c r="DH21" s="42"/>
-      <c r="DI21" s="42"/>
-      <c r="DJ21" s="42"/>
-      <c r="DK21" s="42"/>
-      <c r="DL21" s="42"/>
-      <c r="DM21" s="42"/>
-      <c r="DN21" s="42"/>
-      <c r="DO21" s="42"/>
-      <c r="DP21" s="42"/>
-      <c r="DQ21" s="42"/>
-      <c r="DR21" s="42"/>
-      <c r="DS21" s="42"/>
-      <c r="DT21" s="42"/>
-      <c r="DU21" s="42"/>
-      <c r="DV21" s="42"/>
-      <c r="DW21" s="42"/>
-      <c r="DX21" s="42"/>
-      <c r="DY21" s="42"/>
-      <c r="DZ21" s="42"/>
-      <c r="EA21" s="42"/>
-      <c r="EB21" s="42"/>
-      <c r="EC21" s="42"/>
-      <c r="ED21" s="42"/>
-      <c r="EE21" s="42"/>
-      <c r="EF21" s="42"/>
-      <c r="EG21" s="42"/>
-      <c r="EH21" s="42"/>
-      <c r="EI21" s="42"/>
-      <c r="EJ21" s="42"/>
-      <c r="EK21" s="42"/>
-      <c r="EL21" s="42"/>
-      <c r="EM21" s="42"/>
-      <c r="EN21" s="42"/>
-      <c r="EO21" s="42"/>
-      <c r="EP21" s="42"/>
-      <c r="EQ21" s="42"/>
-      <c r="ER21" s="42"/>
-      <c r="ES21" s="42"/>
-      <c r="ET21" s="42"/>
-      <c r="EU21" s="42"/>
-      <c r="EV21" s="42"/>
-      <c r="EW21" s="42"/>
-      <c r="EX21" s="42"/>
-      <c r="EY21" s="42"/>
-      <c r="EZ21" s="42"/>
-      <c r="FA21" s="42"/>
-      <c r="FB21" s="42"/>
-      <c r="FC21" s="42"/>
-      <c r="FD21" s="42"/>
-      <c r="FE21" s="42"/>
-      <c r="FF21" s="42"/>
-      <c r="FG21" s="42"/>
-      <c r="FH21" s="42"/>
-      <c r="FI21" s="42"/>
-      <c r="FJ21" s="42"/>
-      <c r="FK21" s="42"/>
-      <c r="FL21" s="42"/>
-      <c r="FM21" s="42"/>
-      <c r="FN21" s="42"/>
-      <c r="FO21" s="42"/>
-      <c r="FP21" s="42"/>
-      <c r="FQ21" s="42"/>
-      <c r="FR21" s="42"/>
-      <c r="FS21" s="42"/>
-      <c r="FT21" s="42"/>
-      <c r="FU21" s="42"/>
-      <c r="FV21" s="42"/>
-      <c r="FW21" s="42"/>
-      <c r="FX21" s="42"/>
-      <c r="FY21" s="42"/>
-      <c r="FZ21" s="42"/>
-      <c r="GA21" s="42"/>
-      <c r="GB21" s="42"/>
-      <c r="GC21" s="42"/>
-      <c r="GD21" s="42"/>
-      <c r="GE21" s="42"/>
-      <c r="GF21" s="42"/>
-      <c r="GG21" s="42"/>
-      <c r="GH21" s="42"/>
-      <c r="GI21" s="42"/>
-      <c r="GJ21" s="42"/>
-      <c r="GK21" s="42"/>
-      <c r="GL21" s="42"/>
-      <c r="GM21" s="42"/>
-      <c r="GN21" s="42"/>
-      <c r="GO21" s="42"/>
-      <c r="GP21" s="42"/>
-      <c r="GQ21" s="42"/>
-      <c r="GR21" s="42"/>
-      <c r="GS21" s="42"/>
-      <c r="GT21" s="42"/>
-      <c r="GU21" s="42"/>
-      <c r="GV21" s="42"/>
-      <c r="GW21" s="42"/>
-      <c r="GX21" s="42"/>
-      <c r="GY21" s="42"/>
-      <c r="GZ21" s="42"/>
-      <c r="HA21" s="42"/>
-      <c r="HB21" s="42"/>
-      <c r="HC21" s="42"/>
-      <c r="HD21" s="42"/>
-      <c r="HE21" s="42"/>
-      <c r="HF21" s="42"/>
-      <c r="HG21" s="42"/>
-      <c r="HH21" s="42"/>
-      <c r="HI21" s="42"/>
-      <c r="HJ21" s="42"/>
-      <c r="HK21" s="42"/>
-      <c r="HL21" s="42"/>
-      <c r="HM21" s="42"/>
-      <c r="HN21" s="42"/>
-      <c r="HO21" s="42"/>
-      <c r="HP21" s="42"/>
-      <c r="HQ21" s="42"/>
-      <c r="HR21" s="42"/>
-      <c r="HS21" s="42"/>
-      <c r="HT21" s="42"/>
-      <c r="HU21" s="42"/>
-      <c r="HV21" s="42"/>
-      <c r="HW21" s="42"/>
-      <c r="HX21" s="42"/>
-      <c r="HY21" s="42"/>
-      <c r="HZ21" s="42"/>
-      <c r="IA21" s="42"/>
-      <c r="IB21" s="42"/>
-      <c r="IC21" s="42"/>
-      <c r="ID21" s="42"/>
-      <c r="IE21" s="42"/>
-      <c r="IF21" s="42"/>
-      <c r="IG21" s="42"/>
-      <c r="IH21" s="42"/>
-      <c r="II21" s="42"/>
-      <c r="IJ21" s="42"/>
-      <c r="IK21" s="42"/>
-      <c r="IL21" s="42"/>
-      <c r="IM21" s="42"/>
-      <c r="IN21" s="42"/>
-      <c r="IO21" s="42"/>
-      <c r="IP21" s="42"/>
-      <c r="IQ21" s="42"/>
-      <c r="IR21" s="42"/>
-      <c r="IS21" s="42"/>
-      <c r="IT21" s="42"/>
-      <c r="IU21" s="42"/>
-      <c r="IV21" s="42"/>
-      <c r="IW21" s="42"/>
-      <c r="IX21" s="42"/>
-      <c r="IY21" s="42"/>
-      <c r="IZ21" s="42"/>
-      <c r="JA21" s="42"/>
-      <c r="JB21" s="42"/>
-      <c r="JC21" s="42"/>
-      <c r="JD21" s="42"/>
-      <c r="JE21" s="42"/>
-      <c r="JF21" s="42"/>
-      <c r="JG21" s="42"/>
-      <c r="JH21" s="42"/>
-      <c r="JI21" s="42"/>
-      <c r="JJ21" s="42"/>
-      <c r="JK21" s="42"/>
-      <c r="JL21" s="42"/>
-      <c r="JM21" s="42"/>
-      <c r="JN21" s="42"/>
+      <c r="O21" s="43"/>
+      <c r="P21" s="43"/>
+      <c r="Q21" s="43"/>
+      <c r="R21" s="43"/>
+      <c r="S21" s="43"/>
+      <c r="T21" s="43"/>
+      <c r="U21" s="43"/>
+      <c r="V21" s="43"/>
+      <c r="W21" s="43"/>
+      <c r="X21" s="43"/>
+      <c r="Y21" s="43"/>
+      <c r="Z21" s="43"/>
+      <c r="AA21" s="43"/>
+      <c r="AB21" s="43"/>
+      <c r="AC21" s="43"/>
+      <c r="AD21" s="43"/>
+      <c r="AE21" s="43"/>
+      <c r="AF21" s="43"/>
+      <c r="AG21" s="43"/>
+      <c r="AH21" s="43"/>
+      <c r="AI21" s="43"/>
+      <c r="AJ21" s="43"/>
+      <c r="AK21" s="43"/>
+      <c r="AL21" s="43"/>
+      <c r="AM21" s="43"/>
+      <c r="AN21" s="43"/>
+      <c r="AO21" s="43"/>
+      <c r="AP21" s="43"/>
+      <c r="AQ21" s="43"/>
+      <c r="AR21" s="43"/>
+      <c r="AS21" s="43"/>
+      <c r="AT21" s="43"/>
+      <c r="AU21" s="43"/>
+      <c r="AV21" s="43"/>
+      <c r="AW21" s="43"/>
+      <c r="AX21" s="43"/>
+      <c r="AY21" s="43"/>
+      <c r="AZ21" s="43"/>
+      <c r="BA21" s="43"/>
+      <c r="BB21" s="43"/>
+      <c r="BC21" s="43"/>
+      <c r="BD21" s="43"/>
+      <c r="BE21" s="43"/>
+      <c r="BF21" s="43"/>
+      <c r="BG21" s="43"/>
+      <c r="BH21" s="43"/>
+      <c r="BI21" s="43"/>
+      <c r="BJ21" s="43"/>
+      <c r="BK21" s="43"/>
+      <c r="BL21" s="43"/>
+      <c r="BM21" s="43"/>
+      <c r="BN21" s="43"/>
+      <c r="BO21" s="43"/>
+      <c r="BP21" s="43"/>
+      <c r="BQ21" s="43"/>
+      <c r="BR21" s="43"/>
+      <c r="BS21" s="43"/>
+      <c r="BT21" s="43"/>
+      <c r="BU21" s="43"/>
+      <c r="BV21" s="43"/>
+      <c r="BW21" s="43"/>
+      <c r="BX21" s="43"/>
+      <c r="BY21" s="43"/>
+      <c r="BZ21" s="43"/>
+      <c r="CA21" s="43"/>
+      <c r="CB21" s="43"/>
+      <c r="CC21" s="43"/>
+      <c r="CD21" s="43"/>
+      <c r="CE21" s="43"/>
+      <c r="CF21" s="43"/>
+      <c r="CG21" s="43"/>
+      <c r="CH21" s="43"/>
+      <c r="CI21" s="43"/>
+      <c r="CJ21" s="43"/>
+      <c r="CK21" s="43"/>
+      <c r="CL21" s="43"/>
+      <c r="CM21" s="43"/>
+      <c r="CN21" s="43"/>
+      <c r="CO21" s="43"/>
+      <c r="CP21" s="43"/>
+      <c r="CQ21" s="43"/>
+      <c r="CR21" s="43"/>
+      <c r="CS21" s="43"/>
+      <c r="CT21" s="43"/>
+      <c r="CU21" s="43"/>
+      <c r="CV21" s="43"/>
+      <c r="CW21" s="43"/>
+      <c r="CX21" s="43"/>
+      <c r="CY21" s="43"/>
+      <c r="CZ21" s="43"/>
+      <c r="DA21" s="43"/>
+      <c r="DB21" s="43"/>
+      <c r="DC21" s="43"/>
+      <c r="DD21" s="43"/>
+      <c r="DE21" s="43"/>
+      <c r="DF21" s="43"/>
+      <c r="DG21" s="43"/>
+      <c r="DH21" s="43"/>
+      <c r="DI21" s="43"/>
+      <c r="DJ21" s="43"/>
+      <c r="DK21" s="43"/>
+      <c r="DL21" s="43"/>
+      <c r="DM21" s="43"/>
+      <c r="DN21" s="43"/>
+      <c r="DO21" s="43"/>
+      <c r="DP21" s="43"/>
+      <c r="DQ21" s="43"/>
+      <c r="DR21" s="43"/>
+      <c r="DS21" s="43"/>
+      <c r="DT21" s="43"/>
+      <c r="DU21" s="43"/>
+      <c r="DV21" s="43"/>
+      <c r="DW21" s="43"/>
+      <c r="DX21" s="43"/>
+      <c r="DY21" s="43"/>
+      <c r="DZ21" s="43"/>
+      <c r="EA21" s="43"/>
+      <c r="EB21" s="43"/>
+      <c r="EC21" s="43"/>
+      <c r="ED21" s="43"/>
+      <c r="EE21" s="43"/>
+      <c r="EF21" s="43"/>
+      <c r="EG21" s="43"/>
+      <c r="EH21" s="43"/>
+      <c r="EI21" s="43"/>
+      <c r="EJ21" s="43"/>
+      <c r="EK21" s="43"/>
+      <c r="EL21" s="43"/>
+      <c r="EM21" s="43"/>
+      <c r="EN21" s="43"/>
+      <c r="EO21" s="43"/>
+      <c r="EP21" s="43"/>
+      <c r="EQ21" s="43"/>
+      <c r="ER21" s="43"/>
+      <c r="ES21" s="43"/>
+      <c r="ET21" s="43"/>
+      <c r="EU21" s="43"/>
+      <c r="EV21" s="43"/>
+      <c r="EW21" s="43"/>
+      <c r="EX21" s="43"/>
+      <c r="EY21" s="43"/>
+      <c r="EZ21" s="43"/>
+      <c r="FA21" s="43"/>
+      <c r="FB21" s="43"/>
+      <c r="FC21" s="43"/>
+      <c r="FD21" s="43"/>
+      <c r="FE21" s="43"/>
+      <c r="FF21" s="43"/>
+      <c r="FG21" s="43"/>
+      <c r="FH21" s="43"/>
+      <c r="FI21" s="43"/>
+      <c r="FJ21" s="43"/>
+      <c r="FK21" s="43"/>
+      <c r="FL21" s="43"/>
+      <c r="FM21" s="43"/>
+      <c r="FN21" s="43"/>
+      <c r="FO21" s="43"/>
+      <c r="FP21" s="43"/>
+      <c r="FQ21" s="43"/>
+      <c r="FR21" s="43"/>
+      <c r="FS21" s="43"/>
+      <c r="FT21" s="43"/>
+      <c r="FU21" s="43"/>
+      <c r="FV21" s="43"/>
+      <c r="FW21" s="43"/>
+      <c r="FX21" s="43"/>
+      <c r="FY21" s="43"/>
+      <c r="FZ21" s="43"/>
+      <c r="GA21" s="43"/>
+      <c r="GB21" s="43"/>
+      <c r="GC21" s="43"/>
+      <c r="GD21" s="43"/>
+      <c r="GE21" s="43"/>
+      <c r="GF21" s="43"/>
+      <c r="GG21" s="43"/>
+      <c r="GH21" s="43"/>
+      <c r="GI21" s="43"/>
+      <c r="GJ21" s="43"/>
+      <c r="GK21" s="43"/>
+      <c r="GL21" s="43"/>
+      <c r="GM21" s="43"/>
+      <c r="GN21" s="43"/>
+      <c r="GO21" s="43"/>
+      <c r="GP21" s="43"/>
+      <c r="GQ21" s="43"/>
+      <c r="GR21" s="43"/>
+      <c r="GS21" s="43"/>
+      <c r="GT21" s="43"/>
+      <c r="GU21" s="43"/>
+      <c r="GV21" s="43"/>
+      <c r="GW21" s="43"/>
+      <c r="GX21" s="43"/>
+      <c r="GY21" s="43"/>
+      <c r="GZ21" s="43"/>
+      <c r="HA21" s="43"/>
+      <c r="HB21" s="43"/>
+      <c r="HC21" s="43"/>
+      <c r="HD21" s="43"/>
+      <c r="HE21" s="43"/>
+      <c r="HF21" s="43"/>
+      <c r="HG21" s="43"/>
+      <c r="HH21" s="43"/>
+      <c r="HI21" s="43"/>
+      <c r="HJ21" s="43"/>
+      <c r="HK21" s="43"/>
+      <c r="HL21" s="43"/>
+      <c r="HM21" s="43"/>
+      <c r="HN21" s="43"/>
+      <c r="HO21" s="43"/>
+      <c r="HP21" s="43"/>
+      <c r="HQ21" s="43"/>
+      <c r="HR21" s="43"/>
+      <c r="HS21" s="43"/>
+      <c r="HT21" s="43"/>
+      <c r="HU21" s="43"/>
+      <c r="HV21" s="43"/>
+      <c r="HW21" s="43"/>
+      <c r="HX21" s="43"/>
+      <c r="HY21" s="43"/>
+      <c r="HZ21" s="43"/>
+      <c r="IA21" s="43"/>
+      <c r="IB21" s="43"/>
+      <c r="IC21" s="43"/>
+      <c r="ID21" s="43"/>
+      <c r="IE21" s="43"/>
+      <c r="IF21" s="43"/>
+      <c r="IG21" s="43"/>
+      <c r="IH21" s="43"/>
+      <c r="II21" s="43"/>
+      <c r="IJ21" s="43"/>
+      <c r="IK21" s="43"/>
+      <c r="IL21" s="43"/>
+      <c r="IM21" s="43"/>
+      <c r="IN21" s="43"/>
+      <c r="IO21" s="43"/>
+      <c r="IP21" s="43"/>
+      <c r="IQ21" s="43"/>
+      <c r="IR21" s="43"/>
+      <c r="IS21" s="43"/>
+      <c r="IT21" s="43"/>
+      <c r="IU21" s="43"/>
+      <c r="IV21" s="43"/>
+      <c r="IW21" s="43"/>
+      <c r="IX21" s="43"/>
+      <c r="IY21" s="43"/>
+      <c r="IZ21" s="43"/>
+      <c r="JA21" s="43"/>
+      <c r="JB21" s="43"/>
+      <c r="JC21" s="43"/>
+      <c r="JD21" s="43"/>
+      <c r="JE21" s="43"/>
+      <c r="JF21" s="43"/>
+      <c r="JG21" s="43"/>
+      <c r="JH21" s="43"/>
+      <c r="JI21" s="43"/>
+      <c r="JJ21" s="43"/>
+      <c r="JK21" s="43"/>
+      <c r="JL21" s="43"/>
+      <c r="JM21" s="43"/>
+      <c r="JN21" s="43"/>
     </row>
     <row r="22" ht="42.75">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="44" t="s">
         <v>172</v>
       </c>
-      <c r="B22" s="43" t="s">
+      <c r="B22" s="44" t="s">
         <v>78</v>
       </c>
-      <c r="C22" s="43" t="s">
+      <c r="C22" s="44" t="s">
         <v>104</v>
       </c>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="44" t="s">
         <v>173</v>
       </c>
-      <c r="E22" s="43" t="s">
+      <c r="E22" s="44" t="s">
         <v>174</v>
       </c>
-      <c r="F22" s="44" t="s">
+      <c r="F22" s="45" t="s">
         <v>107</v>
       </c>
-      <c r="G22" s="43" t="s">
+      <c r="G22" s="44" t="s">
         <v>175</v>
       </c>
-      <c r="H22" s="43" t="s">
+      <c r="H22" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="I22" s="45" t="s">
+      <c r="I22" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="J22" s="43" t="s">
+      <c r="J22" s="44" t="s">
         <v>177</v>
       </c>
-      <c r="K22" s="46">
+      <c r="K22" s="47">
         <v>2010</v>
       </c>
-      <c r="L22" s="46" t="s">
+      <c r="L22" s="47" t="s">
         <v>178</v>
       </c>
-      <c r="M22" s="43"/>
-      <c r="N22" s="47" t="s">
+      <c r="M22" s="44"/>
+      <c r="N22" s="48" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="23" s="16" customFormat="1" ht="25.5">
-      <c r="A23" s="43" t="s">
+      <c r="A23" s="44" t="s">
         <v>172</v>
       </c>
-      <c r="B23" s="43" t="s">
+      <c r="B23" s="44" t="s">
         <v>78</v>
       </c>
-      <c r="C23" s="43" t="s">
+      <c r="C23" s="44" t="s">
         <v>154</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="44" t="s">
         <v>180</v>
       </c>
-      <c r="E23" s="46" t="s">
+      <c r="E23" s="47" t="s">
         <v>181</v>
       </c>
-      <c r="F23" s="44" t="s">
+      <c r="F23" s="45" t="s">
         <v>107</v>
       </c>
-      <c r="G23" s="43"/>
-      <c r="H23" s="43" t="s">
+      <c r="G23" s="44"/>
+      <c r="H23" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="I23" s="48" t="s">
+      <c r="I23" s="49" t="s">
         <v>182</v>
       </c>
-      <c r="J23" s="43" t="s">
+      <c r="J23" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="K23" s="46">
+      <c r="K23" s="47">
         <v>2010</v>
       </c>
-      <c r="L23" s="46" t="s">
+      <c r="L23" s="47" t="s">
         <v>178</v>
       </c>
-      <c r="M23" s="43"/>
-      <c r="N23" s="49" t="s">
+      <c r="M23" s="44"/>
+      <c r="N23" s="50" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="24" ht="28.5">
-      <c r="A24" s="43" t="s">
+      <c r="A24" s="44" t="s">
         <v>172</v>
       </c>
-      <c r="B24" s="43" t="s">
+      <c r="B24" s="44" t="s">
         <v>78</v>
       </c>
-      <c r="C24" s="43" t="s">
+      <c r="C24" s="44" t="s">
         <v>154</v>
       </c>
-      <c r="D24" s="43" t="s">
+      <c r="D24" s="44" t="s">
         <v>184</v>
       </c>
-      <c r="E24" s="43" t="s">
+      <c r="E24" s="44" t="s">
         <v>184</v>
       </c>
-      <c r="F24" s="44" t="s">
+      <c r="F24" s="45" t="s">
         <v>107</v>
       </c>
-      <c r="G24" s="43"/>
-      <c r="H24" s="43" t="s">
+      <c r="G24" s="44"/>
+      <c r="H24" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="I24" s="50" t="s">
+      <c r="I24" s="51" t="s">
         <v>185</v>
       </c>
-      <c r="J24" s="43" t="s">
+      <c r="J24" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="K24" s="46">
+      <c r="K24" s="47">
         <v>2010</v>
       </c>
-      <c r="L24" s="46" t="s">
+      <c r="L24" s="47" t="s">
         <v>178</v>
       </c>
-      <c r="M24" s="43"/>
-      <c r="N24" s="47" t="s">
+      <c r="M24" s="44"/>
+      <c r="N24" s="48" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="25" ht="25.5">
-      <c r="A25" s="51" t="s">
+      <c r="A25" s="52" t="s">
         <v>186</v>
       </c>
-      <c r="B25" s="51" t="s">
+      <c r="B25" s="52" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="51" t="s">
+      <c r="C25" s="52" t="s">
         <v>187</v>
       </c>
-      <c r="D25" s="51" t="s">
+      <c r="D25" s="52" t="s">
         <v>188</v>
       </c>
-      <c r="E25" s="51" t="s">
+      <c r="E25" s="52" t="s">
         <v>189</v>
       </c>
-      <c r="F25" s="52" t="s">
+      <c r="F25" s="53" t="s">
         <v>190</v>
       </c>
-      <c r="G25" s="51"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="53" t="s">
+      <c r="G25" s="52"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="54" t="s">
         <v>191</v>
       </c>
-      <c r="J25" s="51"/>
-      <c r="K25" s="51">
+      <c r="J25" s="52"/>
+      <c r="K25" s="52">
         <v>2016</v>
       </c>
-      <c r="L25" s="51" t="s">
+      <c r="L25" s="52" t="s">
         <v>192</v>
       </c>
-      <c r="M25" s="51"/>
+      <c r="M25" s="52"/>
       <c r="N25" s="25"/>
     </row>
     <row r="26" ht="25.5">
-      <c r="A26" s="51" t="s">
+      <c r="A26" s="52" t="s">
         <v>186</v>
       </c>
-      <c r="B26" s="51" t="s">
+      <c r="B26" s="52" t="s">
         <v>78</v>
       </c>
-      <c r="C26" s="51" t="s">
+      <c r="C26" s="52" t="s">
         <v>187</v>
       </c>
-      <c r="D26" s="51" t="s">
+      <c r="D26" s="52" t="s">
         <v>193</v>
       </c>
-      <c r="E26" s="51" t="s">
+      <c r="E26" s="52" t="s">
         <v>189</v>
       </c>
-      <c r="F26" s="52" t="s">
+      <c r="F26" s="53" t="s">
         <v>194</v>
       </c>
-      <c r="G26" s="51"/>
-      <c r="H26" s="51"/>
-      <c r="I26" s="54"/>
-      <c r="J26" s="55"/>
-      <c r="K26" s="51"/>
-      <c r="L26" s="51"/>
-      <c r="M26" s="51"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="55"/>
+      <c r="J26" s="56"/>
+      <c r="K26" s="52"/>
+      <c r="L26" s="52"/>
+      <c r="M26" s="52"/>
       <c r="N26" s="25"/>
     </row>
     <row r="27" ht="25.5">
-      <c r="A27" s="51" t="s">
+      <c r="A27" s="52" t="s">
         <v>186</v>
       </c>
-      <c r="B27" s="51" t="s">
+      <c r="B27" s="52" t="s">
         <v>78</v>
       </c>
-      <c r="C27" s="51" t="s">
+      <c r="C27" s="52" t="s">
         <v>195</v>
       </c>
-      <c r="D27" s="51" t="s">
+      <c r="D27" s="52" t="s">
         <v>196</v>
       </c>
-      <c r="E27" s="51" t="s">
+      <c r="E27" s="52" t="s">
         <v>197</v>
       </c>
-      <c r="F27" s="51" t="s">
+      <c r="F27" s="52" t="s">
         <v>198</v>
       </c>
-      <c r="G27" s="51"/>
-      <c r="H27" s="51"/>
-      <c r="I27" s="53" t="s">
+      <c r="G27" s="52"/>
+      <c r="H27" s="52"/>
+      <c r="I27" s="54" t="s">
         <v>199</v>
       </c>
-      <c r="J27" s="56"/>
-      <c r="K27" s="51"/>
-      <c r="L27" s="51"/>
-      <c r="M27" s="51"/>
+      <c r="J27" s="57"/>
+      <c r="K27" s="52"/>
+      <c r="L27" s="52"/>
+      <c r="M27" s="52"/>
       <c r="N27" s="25"/>
     </row>
     <row r="28" ht="38.25">
-      <c r="A28" s="51" t="s">
+      <c r="A28" s="52" t="s">
         <v>186</v>
       </c>
-      <c r="B28" s="51" t="s">
+      <c r="B28" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="51" t="s">
+      <c r="C28" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="51" t="s">
+      <c r="D28" s="52" t="s">
         <v>200</v>
       </c>
-      <c r="E28" s="51" t="s">
+      <c r="E28" s="52" t="s">
         <v>201</v>
       </c>
-      <c r="F28" s="57" t="s">
+      <c r="F28" s="58" t="s">
         <v>202</v>
       </c>
-      <c r="G28" s="51" t="s">
+      <c r="G28" s="52" t="s">
         <v>203</v>
       </c>
-      <c r="H28" s="51" t="s">
+      <c r="H28" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="I28" s="58" t="s">
+      <c r="I28" s="59" t="s">
         <v>204</v>
       </c>
-      <c r="J28" s="51" t="s">
+      <c r="J28" s="52" t="s">
         <v>205</v>
       </c>
-      <c r="K28" s="51"/>
-      <c r="L28" s="51" t="s">
+      <c r="K28" s="52"/>
+      <c r="L28" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="M28" s="51"/>
-      <c r="N28" s="59" t="s">
+      <c r="M28" s="52"/>
+      <c r="N28" s="60" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="29" ht="89.25">
-      <c r="A29" s="51" t="s">
+      <c r="A29" s="52" t="s">
         <v>186</v>
       </c>
-      <c r="B29" s="51" t="s">
+      <c r="B29" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="51" t="s">
+      <c r="C29" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="D29" s="51" t="s">
+      <c r="D29" s="52" t="s">
         <v>207</v>
       </c>
-      <c r="E29" s="51" t="s">
+      <c r="E29" s="52" t="s">
         <v>208</v>
       </c>
-      <c r="F29" s="51" t="s">
+      <c r="F29" s="52" t="s">
         <v>82</v>
       </c>
-      <c r="G29" s="51" t="s">
+      <c r="G29" s="52" t="s">
         <v>209</v>
       </c>
-      <c r="H29" s="51" t="s">
+      <c r="H29" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="I29" s="58" t="s">
+      <c r="I29" s="59" t="s">
         <v>85</v>
       </c>
-      <c r="J29" s="51" t="s">
+      <c r="J29" s="52" t="s">
         <v>210</v>
       </c>
-      <c r="K29" s="51" t="s">
+      <c r="K29" s="52" t="s">
         <v>93</v>
       </c>
-      <c r="L29" s="51" t="s">
+      <c r="L29" s="52" t="s">
         <v>24</v>
       </c>
-      <c r="M29" s="51"/>
-      <c r="N29" s="59" t="s">
+      <c r="M29" s="52"/>
+      <c r="N29" s="60" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="30" ht="25.5">
-      <c r="A30" s="60" t="s">
+      <c r="A30" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B30" s="60" t="s">
+      <c r="B30" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="C30" s="60" t="s">
+      <c r="C30" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="D30" s="60" t="s">
+      <c r="D30" s="61" t="s">
         <v>212</v>
       </c>
-      <c r="E30" s="60" t="s">
+      <c r="E30" s="61" t="s">
         <v>213</v>
       </c>
-      <c r="F30" s="61"/>
-      <c r="G30" s="60"/>
-      <c r="H30" s="60"/>
-      <c r="I30" s="62" t="s">
+      <c r="F30" s="62"/>
+      <c r="G30" s="61"/>
+      <c r="H30" s="61"/>
+      <c r="I30" s="63" t="s">
         <v>214</v>
       </c>
-      <c r="J30" s="63"/>
-      <c r="K30" s="60"/>
-      <c r="L30" s="60" t="s">
+      <c r="J30" s="64"/>
+      <c r="K30" s="61"/>
+      <c r="L30" s="61" t="s">
         <v>215</v>
       </c>
-      <c r="M30" s="60"/>
+      <c r="M30" s="61"/>
       <c r="N30" s="36"/>
     </row>
     <row r="31" ht="25.5">
-      <c r="A31" s="60" t="s">
+      <c r="A31" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B31" s="60" t="s">
+      <c r="B31" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="C31" s="60" t="s">
+      <c r="C31" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="D31" s="60" t="s">
+      <c r="D31" s="61" t="s">
         <v>216</v>
       </c>
-      <c r="E31" s="60" t="s">
+      <c r="E31" s="61" t="s">
         <v>213</v>
       </c>
-      <c r="F31" s="61"/>
-      <c r="G31" s="60"/>
-      <c r="H31" s="60"/>
-      <c r="I31" s="62" t="s">
+      <c r="F31" s="62"/>
+      <c r="G31" s="61"/>
+      <c r="H31" s="61"/>
+      <c r="I31" s="63" t="s">
         <v>217</v>
       </c>
-      <c r="J31" s="60"/>
-      <c r="K31" s="60"/>
-      <c r="L31" s="60"/>
-      <c r="M31" s="60"/>
+      <c r="J31" s="61"/>
+      <c r="K31" s="61"/>
+      <c r="L31" s="61"/>
+      <c r="M31" s="61"/>
       <c r="N31" s="36"/>
     </row>
     <row r="32" ht="25.5">
-      <c r="A32" s="60" t="s">
+      <c r="A32" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B32" s="60" t="s">
+      <c r="B32" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="C32" s="60" t="s">
+      <c r="C32" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="D32" s="60" t="s">
+      <c r="D32" s="61" t="s">
         <v>218</v>
       </c>
-      <c r="E32" s="60" t="s">
+      <c r="E32" s="61" t="s">
         <v>213</v>
       </c>
-      <c r="F32" s="61"/>
-      <c r="G32" s="60"/>
-      <c r="H32" s="60"/>
-      <c r="I32" s="62" t="s">
+      <c r="F32" s="62"/>
+      <c r="G32" s="61"/>
+      <c r="H32" s="61"/>
+      <c r="I32" s="63" t="s">
         <v>214</v>
       </c>
-      <c r="J32" s="63"/>
-      <c r="K32" s="60"/>
-      <c r="L32" s="60" t="s">
+      <c r="J32" s="64"/>
+      <c r="K32" s="61"/>
+      <c r="L32" s="61" t="s">
         <v>215</v>
       </c>
-      <c r="M32" s="60"/>
+      <c r="M32" s="61"/>
       <c r="N32" s="36"/>
     </row>
     <row r="33" ht="25.5">
-      <c r="A33" s="60" t="s">
+      <c r="A33" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B33" s="60" t="s">
+      <c r="B33" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="60" t="s">
+      <c r="C33" s="61" t="s">
         <v>154</v>
       </c>
-      <c r="D33" s="60" t="s">
+      <c r="D33" s="61" t="s">
         <v>219</v>
       </c>
-      <c r="E33" s="60"/>
-      <c r="F33" s="61" t="s">
+      <c r="E33" s="61"/>
+      <c r="F33" s="62" t="s">
         <v>220</v>
       </c>
-      <c r="G33" s="60"/>
-      <c r="H33" s="60"/>
-      <c r="I33" s="64"/>
-      <c r="J33" s="60"/>
-      <c r="K33" s="60"/>
-      <c r="L33" s="60"/>
-      <c r="M33" s="60"/>
+      <c r="G33" s="61"/>
+      <c r="H33" s="61"/>
+      <c r="I33" s="65"/>
+      <c r="J33" s="61"/>
+      <c r="K33" s="61"/>
+      <c r="L33" s="61"/>
+      <c r="M33" s="61"/>
       <c r="N33" s="36"/>
     </row>
     <row r="34" ht="25.5">
-      <c r="A34" s="60" t="s">
+      <c r="A34" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B34" s="60" t="s">
+      <c r="B34" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="C34" s="60" t="s">
+      <c r="C34" s="61" t="s">
         <v>195</v>
       </c>
-      <c r="D34" s="60" t="s">
+      <c r="D34" s="61" t="s">
         <v>221</v>
       </c>
-      <c r="E34" s="60" t="s">
+      <c r="E34" s="61" t="s">
         <v>213</v>
       </c>
-      <c r="F34" s="61"/>
-      <c r="G34" s="60"/>
-      <c r="H34" s="60"/>
-      <c r="I34" s="65"/>
-      <c r="J34" s="60"/>
-      <c r="K34" s="60"/>
-      <c r="L34" s="60"/>
-      <c r="M34" s="60"/>
+      <c r="F34" s="62"/>
+      <c r="G34" s="61"/>
+      <c r="H34" s="61"/>
+      <c r="I34" s="66"/>
+      <c r="J34" s="61"/>
+      <c r="K34" s="61"/>
+      <c r="L34" s="61"/>
+      <c r="M34" s="61"/>
       <c r="N34" s="36"/>
     </row>
     <row r="35" ht="38.25">
-      <c r="A35" s="60" t="s">
+      <c r="A35" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B35" s="60" t="s">
+      <c r="B35" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="C35" s="60" t="s">
+      <c r="C35" s="61" t="s">
         <v>195</v>
       </c>
-      <c r="D35" s="60" t="s">
+      <c r="D35" s="61" t="s">
         <v>222</v>
       </c>
-      <c r="E35" s="60" t="s">
+      <c r="E35" s="61" t="s">
         <v>213</v>
       </c>
-      <c r="F35" s="61" t="s">
+      <c r="F35" s="62" t="s">
         <v>223</v>
       </c>
-      <c r="G35" s="60"/>
-      <c r="H35" s="60"/>
-      <c r="I35" s="62" t="s">
+      <c r="G35" s="61"/>
+      <c r="H35" s="61"/>
+      <c r="I35" s="63" t="s">
         <v>224</v>
       </c>
-      <c r="J35" s="60"/>
-      <c r="K35" s="60"/>
-      <c r="L35" s="60"/>
-      <c r="M35" s="60"/>
+      <c r="J35" s="61"/>
+      <c r="K35" s="61"/>
+      <c r="L35" s="61"/>
+      <c r="M35" s="61"/>
       <c r="N35" s="36"/>
     </row>
     <row r="36" ht="38.25">
-      <c r="A36" s="60" t="s">
+      <c r="A36" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B36" s="60" t="s">
+      <c r="B36" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="C36" s="60" t="s">
+      <c r="C36" s="61" t="s">
         <v>225</v>
       </c>
-      <c r="D36" s="60" t="s">
+      <c r="D36" s="61" t="s">
         <v>226</v>
       </c>
-      <c r="E36" s="60" t="s">
+      <c r="E36" s="61" t="s">
         <v>227</v>
       </c>
-      <c r="F36" s="61" t="s">
+      <c r="F36" s="62" t="s">
         <v>228</v>
       </c>
-      <c r="G36" s="60"/>
-      <c r="H36" s="60"/>
-      <c r="I36" s="62" t="s">
+      <c r="G36" s="61"/>
+      <c r="H36" s="61"/>
+      <c r="I36" s="63" t="s">
         <v>229</v>
       </c>
-      <c r="J36" s="60"/>
-      <c r="K36" s="60"/>
-      <c r="L36" s="60" t="s">
+      <c r="J36" s="61"/>
+      <c r="K36" s="61"/>
+      <c r="L36" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="M36" s="60"/>
+      <c r="M36" s="61"/>
       <c r="N36" s="36"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="60" t="s">
+      <c r="A37" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B37" s="60" t="s">
+      <c r="B37" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="60" t="s">
+      <c r="C37" s="61" t="s">
         <v>230</v>
       </c>
-      <c r="D37" s="60" t="s">
+      <c r="D37" s="61" t="s">
         <v>231</v>
       </c>
-      <c r="E37" s="60" t="s">
+      <c r="E37" s="61" t="s">
         <v>213</v>
       </c>
-      <c r="F37" s="60"/>
-      <c r="G37" s="60"/>
-      <c r="H37" s="60"/>
-      <c r="I37" s="66"/>
-      <c r="J37" s="60"/>
-      <c r="K37" s="60"/>
-      <c r="L37" s="60"/>
-      <c r="M37" s="60"/>
-      <c r="N37" s="60" t="s">
+      <c r="F37" s="61"/>
+      <c r="G37" s="61"/>
+      <c r="H37" s="61"/>
+      <c r="I37" s="67"/>
+      <c r="J37" s="61"/>
+      <c r="K37" s="61"/>
+      <c r="L37" s="61"/>
+      <c r="M37" s="61"/>
+      <c r="N37" s="61" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="38" ht="51">
-      <c r="A38" s="60" t="s">
+      <c r="A38" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B38" s="60" t="s">
+      <c r="B38" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="60" t="s">
+      <c r="C38" s="61" t="s">
         <v>230</v>
       </c>
-      <c r="D38" s="60" t="s">
+      <c r="D38" s="61" t="s">
         <v>233</v>
       </c>
-      <c r="E38" s="60" t="s">
+      <c r="E38" s="61" t="s">
         <v>213</v>
       </c>
-      <c r="F38" s="60"/>
-      <c r="G38" s="60"/>
-      <c r="H38" s="60"/>
-      <c r="I38" s="66"/>
-      <c r="J38" s="60"/>
-      <c r="K38" s="60"/>
-      <c r="L38" s="60"/>
-      <c r="M38" s="60"/>
-      <c r="N38" s="60" t="s">
+      <c r="F38" s="61"/>
+      <c r="G38" s="61"/>
+      <c r="H38" s="61"/>
+      <c r="I38" s="67"/>
+      <c r="J38" s="61"/>
+      <c r="K38" s="61"/>
+      <c r="L38" s="61"/>
+      <c r="M38" s="61"/>
+      <c r="N38" s="61" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="39" ht="51">
-      <c r="A39" s="60" t="s">
+      <c r="A39" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B39" s="60" t="s">
+      <c r="B39" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="C39" s="60" t="s">
+      <c r="C39" s="61" t="s">
         <v>234</v>
       </c>
-      <c r="D39" s="60" t="s">
+      <c r="D39" s="61" t="s">
         <v>235</v>
       </c>
-      <c r="E39" s="60" t="s">
+      <c r="E39" s="61" t="s">
         <v>236</v>
       </c>
-      <c r="F39" s="67" t="s">
+      <c r="F39" s="68" t="s">
         <v>237</v>
       </c>
-      <c r="G39" s="60"/>
-      <c r="H39" s="60"/>
-      <c r="I39" s="66"/>
-      <c r="J39" s="60"/>
-      <c r="K39" s="60"/>
-      <c r="L39" s="60"/>
-      <c r="M39" s="60"/>
-      <c r="N39" s="60" t="s">
+      <c r="G39" s="61"/>
+      <c r="H39" s="61"/>
+      <c r="I39" s="67"/>
+      <c r="J39" s="61"/>
+      <c r="K39" s="61"/>
+      <c r="L39" s="61"/>
+      <c r="M39" s="61"/>
+      <c r="N39" s="61" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="40" s="10" customFormat="1" ht="25.5">
-      <c r="A40" s="60" t="s">
+      <c r="A40" s="61" t="s">
         <v>211</v>
       </c>
-      <c r="B40" s="60" t="s">
+      <c r="B40" s="61" t="s">
         <v>36</v>
       </c>
-      <c r="C40" s="60" t="s">
+      <c r="C40" s="61" t="s">
         <v>68</v>
       </c>
-      <c r="D40" s="60" t="s">
+      <c r="D40" s="61" t="s">
         <v>238</v>
       </c>
-      <c r="E40" s="60" t="s">
+      <c r="E40" s="61" t="s">
         <v>213</v>
       </c>
-      <c r="F40" s="60"/>
-      <c r="G40" s="60"/>
-      <c r="H40" s="60"/>
-      <c r="I40" s="66"/>
-      <c r="J40" s="60"/>
-      <c r="K40" s="60"/>
-      <c r="L40" s="60"/>
-      <c r="M40" s="60"/>
-      <c r="N40" s="60" t="s">
+      <c r="F40" s="61"/>
+      <c r="G40" s="61"/>
+      <c r="H40" s="61"/>
+      <c r="I40" s="67"/>
+      <c r="J40" s="61"/>
+      <c r="K40" s="61"/>
+      <c r="L40" s="61"/>
+      <c r="M40" s="61"/>
+      <c r="N40" s="61" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="41" ht="14.25">
-      <c r="A41" s="68" t="s">
+      <c r="A41" s="69" t="s">
         <v>239</v>
       </c>
-      <c r="B41" s="68" t="s">
+      <c r="B41" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="C41" s="68" t="s">
+      <c r="C41" s="69" t="s">
         <v>89</v>
       </c>
-      <c r="D41" s="68" t="s">
+      <c r="D41" s="69" t="s">
         <v>240</v>
       </c>
-      <c r="E41" s="68" t="s">
+      <c r="E41" s="69" t="s">
         <v>241</v>
       </c>
-      <c r="F41" s="68"/>
-      <c r="G41" s="68" t="s">
+      <c r="F41" s="69"/>
+      <c r="G41" s="69" t="s">
         <v>242</v>
       </c>
-      <c r="H41" s="68" t="s">
+      <c r="H41" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="I41" s="69"/>
-      <c r="J41" s="68"/>
-      <c r="K41" s="68"/>
-      <c r="L41" s="68"/>
-      <c r="M41" s="68" t="s">
+      <c r="I41" s="70"/>
+      <c r="J41" s="69"/>
+      <c r="K41" s="69"/>
+      <c r="L41" s="69"/>
+      <c r="M41" s="69" t="s">
         <v>140</v>
       </c>
-      <c r="N41" s="68"/>
+      <c r="N41" s="69"/>
     </row>
     <row r="42" ht="14.25">
       <c r="A42" s="1"/>
-      <c r="M42" s="70"/>
-      <c r="N42" s="70"/>
+      <c r="M42" s="71"/>
+      <c r="N42" s="71"/>
     </row>
     <row r="43" ht="14.25">
-      <c r="M43" s="70"/>
-      <c r="N43" s="70"/>
+      <c r="M43" s="71"/>
+      <c r="N43" s="71"/>
     </row>
     <row r="44" ht="14.25">
-      <c r="M44" s="70"/>
-      <c r="N44" s="70"/>
+      <c r="M44" s="71"/>
+      <c r="N44" s="71"/>
     </row>
     <row r="45" ht="14.25">
-      <c r="M45" s="70"/>
-      <c r="N45" s="70"/>
+      <c r="M45" s="71"/>
+      <c r="N45" s="71"/>
     </row>
     <row r="46" ht="14.25">
-      <c r="M46" s="70"/>
-      <c r="N46" s="70"/>
+      <c r="M46" s="71"/>
+      <c r="N46" s="71"/>
     </row>
     <row r="47" ht="14.25">
-      <c r="M47" s="70"/>
-      <c r="N47" s="70"/>
+      <c r="M47" s="71"/>
+      <c r="N47" s="71"/>
     </row>
     <row r="48" ht="14.25">
-      <c r="M48" s="70"/>
-      <c r="N48" s="70"/>
+      <c r="M48" s="71"/>
+      <c r="N48" s="71"/>
     </row>
     <row r="49" ht="14.25">
-      <c r="M49" s="70"/>
-      <c r="N49" s="70"/>
+      <c r="M49" s="71"/>
+      <c r="N49" s="71"/>
     </row>
     <row r="50" ht="14.25">
-      <c r="M50" s="70"/>
-      <c r="N50" s="70"/>
+      <c r="M50" s="71"/>
+      <c r="N50" s="71"/>
     </row>
     <row r="51" ht="14.25">
-      <c r="M51" s="70"/>
-      <c r="N51" s="70"/>
+      <c r="M51" s="71"/>
+      <c r="N51" s="71"/>
     </row>
     <row r="52" ht="14.25">
-      <c r="M52" s="70"/>
-      <c r="N52" s="70"/>
+      <c r="M52" s="71"/>
+      <c r="N52" s="71"/>
     </row>
     <row r="53" ht="14.25">
-      <c r="M53" s="70"/>
-      <c r="N53" s="70"/>
+      <c r="M53" s="71"/>
+      <c r="N53" s="71"/>
     </row>
     <row r="54" ht="14.25">
-      <c r="M54" s="70"/>
-      <c r="N54" s="70"/>
+      <c r="M54" s="71"/>
+      <c r="N54" s="71"/>
     </row>
     <row r="55" ht="14.25">
-      <c r="M55" s="70"/>
-      <c r="N55" s="70"/>
+      <c r="M55" s="71"/>
+      <c r="N55" s="71"/>
     </row>
     <row r="56" ht="14.25">
-      <c r="M56" s="70"/>
-      <c r="N56" s="70"/>
+      <c r="M56" s="71"/>
+      <c r="N56" s="71"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N41">
@@ -8644,18 +8649,18 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="72" t="s">
         <v>243</v>
       </c>
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="72" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="2" s="0" customFormat="1" ht="14.25">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="74" t="s">
         <v>245</v>
       </c>
       <c r="C2"/>
@@ -8669,7 +8674,7 @@
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="44" t="s">
         <v>172</v>
       </c>
       <c r="B4" t="s">
@@ -8677,7 +8682,7 @@
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="52" t="s">
         <v>186</v>
       </c>
       <c r="B5" t="s">
@@ -8685,7 +8690,7 @@
       </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="60" t="s">
+      <c r="A6" s="61" t="s">
         <v>211</v>
       </c>
       <c r="B6" t="s">
@@ -8693,7 +8698,7 @@
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="68" t="s">
+      <c r="A7" s="69" t="s">
         <v>239</v>
       </c>
       <c r="B7" t="s">
@@ -8720,19 +8725,19 @@
     <col customWidth="1" min="6" max="6" width="12.8515625"/>
     <col bestFit="1" customWidth="1" min="7" max="7" width="25.78125"/>
     <col bestFit="1" customWidth="1" min="8" max="8" width="21.3515625"/>
-    <col customWidth="1" min="9" max="9" style="74" width="32.7109375"/>
+    <col customWidth="1" min="9" max="9" style="75" width="32.7109375"/>
     <col customWidth="1" min="10" max="10" width="23.57421875"/>
     <col customWidth="1" min="11" max="11" width="44.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" s="71" customFormat="1" ht="25.5">
-      <c r="A1" s="71" t="s">
+    <row r="1" s="72" customFormat="1" ht="25.5">
+      <c r="A1" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="72" t="s">
         <v>251</v>
       </c>
-      <c r="C1" s="71" t="s">
+      <c r="C1" s="72" t="s">
         <v>252</v>
       </c>
       <c r="D1" s="4" t="s">
@@ -8750,48 +8755,48 @@
       <c r="H1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="75" t="s">
+      <c r="I1" s="76" t="s">
         <v>253</v>
       </c>
-      <c r="J1" s="71" t="s">
+      <c r="J1" s="72" t="s">
         <v>254</v>
       </c>
-      <c r="K1" s="71" t="s">
+      <c r="K1" s="72" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" s="76" customFormat="1" ht="28.5">
-      <c r="A2" s="77" t="s">
+    <row r="2" s="77" customFormat="1" ht="28.5">
+      <c r="A2" s="78" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="78" t="s">
+      <c r="B2" s="79" t="s">
         <v>255</v>
       </c>
-      <c r="C2" s="77" t="s">
+      <c r="C2" s="78" t="s">
         <v>256</v>
       </c>
-      <c r="D2" s="78" t="s">
+      <c r="D2" s="79" t="s">
         <v>257</v>
       </c>
-      <c r="E2" s="78" t="s">
+      <c r="E2" s="79" t="s">
         <v>258</v>
       </c>
-      <c r="F2" s="78" t="s">
+      <c r="F2" s="79" t="s">
         <v>259</v>
       </c>
-      <c r="G2" s="76" t="s">
+      <c r="G2" s="77" t="s">
         <v>260</v>
       </c>
-      <c r="H2" s="77" t="s">
+      <c r="H2" s="78" t="s">
         <v>261</v>
       </c>
-      <c r="I2" s="79" t="s">
+      <c r="I2" s="80" t="s">
         <v>262</v>
       </c>
-      <c r="J2" s="76" t="s">
+      <c r="J2" s="77" t="s">
         <v>263</v>
       </c>
-      <c r="K2" s="80" t="s">
+      <c r="K2" s="81" t="s">
         <v>264</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add distance refea and agreste 2010 data
</commit_message>
<xml_diff>
--- a/progress/megatrends_RF.xlsx
+++ b/progress/megatrends_RF.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="270">
   <si>
     <t>Calcul</t>
   </si>
@@ -393,7 +393,7 @@
     <t>https://stats.agriculture.gouv.fr/cartostat/#c=indicator&amp;i=stru_2020_1.nbexpl20&amp;t=A02&amp;view=map11</t>
   </si>
   <si>
-    <t>data_Agreste_Commune.csv</t>
+    <t>data_Agreste_Commune2020.csv</t>
   </si>
   <si>
     <t>02h_get_agreste.R</t>
@@ -429,6 +429,52 @@
     <t>https://stats.agriculture.gouv.fr/cartostat/#c=indicator&amp;i=stru_2020_1.pbs20&amp;t=A02&amp;view=map11</t>
   </si>
   <si>
+    <t xml:space="preserve">Education level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pct_Superieur → Percent of farm holders with higher education.</t>
+  </si>
+  <si>
+    <t>AGRESTE_EDUSUP_PCT_2010</t>
+  </si>
+  <si>
+    <t>https://stats.agriculture.gouv.fr/cartostat/#c=indicator&amp;i=empl1.partformsup10&amp;t=A02&amp;view=map1</t>
+  </si>
+  <si>
+    <t>data_Agreste_Commune2010.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changes in the farmer populations </t>
+  </si>
+  <si>
+    <t xml:space="preserve">farm size</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Average farm size per commune
+</t>
+    </r>
+    <r>
+      <rPr>
+        <color indexed="2"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">OPPOSITE OF Density of farmer</t>
+    </r>
+  </si>
+  <si>
+    <t>AGRESTE_FARMSIZE_HA_2010</t>
+  </si>
+  <si>
+    <t>https://stats.agriculture.gouv.fr/cartostat/#c=indicator&amp;i=raanc2.saumoyaa&amp;s=2010&amp;t=A02&amp;view=map1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Crop rotation</t>
   </si>
   <si>
@@ -454,6 +500,40 @@
   </si>
   <si>
     <t xml:space="preserve">could be calculated per field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distance to a training center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Euclidean distance (in km) from the centroid of each municipality to the centroid of the nearest municipality containing one or more agricultural training centers.</t>
+  </si>
+  <si>
+    <t>MASA</t>
+  </si>
+  <si>
+    <t>REFEA_DIST_KM_2025</t>
+  </si>
+  <si>
+    <t>km</t>
+  </si>
+  <si>
+    <t>https://www.data.gouv.fr/fr/datasets/refea-liste-des-etablissements-proposant-des-formations-agricoles/</t>
+  </si>
+  <si>
+    <t>refea_2025-2026.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2006, 2026</t>
+  </si>
+  <si>
+    <t>coordinates</t>
+  </si>
+  <si>
+    <t>02j_get_refea.R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://enseignement-agricole.opendatasoft.com/explore/dataset/uai_vu1_1_1/export/
+https://enseignement-agricole.opendatasoft.com/explore/dataset/refea-liste-des-etablissements-proposant-des-formations-agricoles-2025-2026/export/</t>
   </si>
   <si>
     <t xml:space="preserve">1. almost</t>
@@ -486,56 +566,6 @@
   <si>
     <t xml:space="preserve">not same commune (3000 mismatch)
 can it be calculated at maille level?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distance to a training center</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Euclidean distance (in km) from the centroid of each municipality to the centroid of the nearest municipality containing one or more agricultural training centers.</t>
-  </si>
-  <si>
-    <t>MASA</t>
-  </si>
-  <si>
-    <t>DIST_TRAIN</t>
-  </si>
-  <si>
-    <t>km</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.data.gouv.fr/fr/datasets/refea-liste-des-etablissements-proposant-des-formations-agricoles/
-https://enseignement-agricole.opendatasoft.com/explore/dataset/uai_vu1_1_1/export/
-https://enseignement-agricole.opendatasoft.com/explore/dataset/refea-liste-des-etablissements-proposant-des-formations-agricoles-2025-2026/export/</t>
-  </si>
-  <si>
-    <t>refea_2025-2026.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2006, 2026</t>
-  </si>
-  <si>
-    <t>coordinates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Education level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pct_Superieur → Percent of farm holders with higher education.</t>
-  </si>
-  <si>
-    <t>https://stats.agriculture.gouv.fr/cartostat/#c=indicator&amp;i=empl1.partformsup10&amp;t=A02&amp;view=map1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Changes in the farmer populations </t>
-  </si>
-  <si>
-    <t xml:space="preserve">farm size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Average farm size per commune</t>
-  </si>
-  <si>
-    <t>https://stats.agriculture.gouv.fr/cartostat/#c=indicator&amp;i=raanc2.saumoyaa&amp;s=2010&amp;t=A02&amp;view=map1</t>
   </si>
   <si>
     <t>Urbanization</t>
@@ -978,14 +1008,13 @@
     </font>
     <font>
       <sz val="10.000000"/>
-      <color indexed="2"/>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <sz val="10.000000"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
+      <color indexed="2"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -1008,7 +1037,8 @@
     <font>
       <sz val="10.000000"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1044,12 +1074,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="-0.249977111117893"/>
-        <bgColor theme="7" tint="-0.249977111117893"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.099978637043366805"/>
         <bgColor theme="2" tint="-0.099978637043366805"/>
       </patternFill>
@@ -1058,6 +1082,12 @@
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor theme="7" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
+        <bgColor theme="7" tint="-0.249977111117893"/>
       </patternFill>
     </fill>
   </fills>
@@ -1073,7 +1103,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="78">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1147,13 +1177,19 @@
     <xf fontId="10" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="11" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf fontId="2" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="11" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="12" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="11" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="12" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1161,28 +1197,6 @@
     </xf>
     <xf fontId="2" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="5" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="8" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="4" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
-    <xf fontId="6" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="12" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="5" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1194,26 +1208,29 @@
       <alignment vertical="center"/>
     </xf>
     <xf fontId="10" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="2" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="5" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="3" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="3" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="4" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="4" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="13" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="13" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="14" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="14" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="9" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="3" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="9" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="3" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf fontId="2" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1234,7 +1251,7 @@
     <xf fontId="6" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="11" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="12" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="5" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1243,37 +1260,38 @@
     <xf fontId="1" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="2" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="5" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="6" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="11" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="12" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="2" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="5" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="6" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="17" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="11" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="5" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="12" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="17" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="13" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6055,10 +6073,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>123</v>
@@ -6066,31 +6084,31 @@
       <c r="E15" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="H15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I15" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="18" t="s">
+      <c r="J15" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="J15" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K15" s="7" t="s">
-        <v>129</v>
+      <c r="K15" s="9">
+        <v>2010</v>
       </c>
       <c r="L15" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="M15" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="N15" s="7" t="s">
-        <v>131</v>
-      </c>
+      <c r="M15" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="N15" s="27"/>
       <c r="O15" s="16"/>
       <c r="P15" s="16"/>
       <c r="Q15" s="16"/>
@@ -6353,48 +6371,46 @@
       <c r="JN15" s="16"/>
     </row>
     <row r="16" s="6" customFormat="1" ht="51">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="B16" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="D16" s="27" t="s">
-        <v>134</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="F16" s="28" t="s">
-        <v>136</v>
-      </c>
-      <c r="G16" s="27" t="s">
-        <v>137</v>
-      </c>
-      <c r="H16" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="I16" s="29" t="s">
-        <v>138</v>
-      </c>
-      <c r="J16" s="28" t="s">
-        <v>139</v>
-      </c>
-      <c r="K16" s="27">
-        <v>2023</v>
-      </c>
-      <c r="L16" s="27" t="s">
-        <v>24</v>
-      </c>
-      <c r="M16" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="N16" s="28" t="s">
-        <v>141</v>
-      </c>
+      <c r="J16" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="K16" s="9">
+        <v>2010</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M16" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="N16" s="10"/>
       <c r="O16" s="10"/>
       <c r="P16" s="10"/>
       <c r="Q16" s="10"/>
@@ -6656,381 +6672,395 @@
       <c r="JM16" s="10"/>
       <c r="JN16" s="10"/>
     </row>
-    <row r="17" s="30" customFormat="1" ht="38.25">
-      <c r="A17" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="B17" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="C17" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>142</v>
-      </c>
-      <c r="E17" s="27" t="s">
-        <v>143</v>
-      </c>
-      <c r="F17" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="G17" s="27" t="s">
-        <v>145</v>
-      </c>
-      <c r="H17" s="27" t="s">
-        <v>146</v>
-      </c>
-      <c r="I17" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="J17" s="33" t="s">
-        <v>148</v>
-      </c>
-      <c r="K17" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="L17" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="M17" s="27"/>
-      <c r="N17" s="16"/>
+    <row r="17" s="6" customFormat="1" ht="38.25">
+      <c r="A17" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="H17" s="7"/>
+      <c r="I17" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="18" s="6" customFormat="1" ht="25.5">
-      <c r="A18" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="B18" s="27" t="s">
+      <c r="A18" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="J18" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="M18" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="E18" s="27" t="s">
+      <c r="N18" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="F18" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27" t="s">
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="10"/>
+      <c r="V18" s="10"/>
+      <c r="W18" s="10"/>
+      <c r="X18" s="10"/>
+      <c r="Y18" s="10"/>
+      <c r="Z18" s="10"/>
+      <c r="AA18" s="10"/>
+      <c r="AB18" s="10"/>
+      <c r="AC18" s="10"/>
+      <c r="AD18" s="10"/>
+      <c r="AE18" s="10"/>
+      <c r="AF18" s="10"/>
+      <c r="AG18" s="10"/>
+      <c r="AH18" s="10"/>
+      <c r="AI18" s="10"/>
+      <c r="AJ18" s="10"/>
+      <c r="AK18" s="10"/>
+      <c r="AL18" s="10"/>
+      <c r="AM18" s="10"/>
+      <c r="AN18" s="10"/>
+      <c r="AO18" s="10"/>
+      <c r="AP18" s="10"/>
+      <c r="AQ18" s="10"/>
+      <c r="AR18" s="10"/>
+      <c r="AS18" s="10"/>
+      <c r="AT18" s="10"/>
+      <c r="AU18" s="10"/>
+      <c r="AV18" s="10"/>
+      <c r="AW18" s="10"/>
+      <c r="AX18" s="10"/>
+      <c r="AY18" s="10"/>
+      <c r="AZ18" s="10"/>
+      <c r="BA18" s="10"/>
+      <c r="BB18" s="10"/>
+      <c r="BC18" s="10"/>
+      <c r="BD18" s="10"/>
+      <c r="BE18" s="10"/>
+      <c r="BF18" s="10"/>
+      <c r="BG18" s="10"/>
+      <c r="BH18" s="10"/>
+      <c r="BI18" s="10"/>
+      <c r="BJ18" s="10"/>
+      <c r="BK18" s="10"/>
+      <c r="BL18" s="10"/>
+      <c r="BM18" s="10"/>
+      <c r="BN18" s="10"/>
+      <c r="BO18" s="10"/>
+      <c r="BP18" s="10"/>
+      <c r="BQ18" s="10"/>
+      <c r="BR18" s="10"/>
+      <c r="BS18" s="10"/>
+      <c r="BT18" s="10"/>
+      <c r="BU18" s="10"/>
+      <c r="BV18" s="10"/>
+      <c r="BW18" s="10"/>
+      <c r="BX18" s="10"/>
+      <c r="BY18" s="10"/>
+      <c r="BZ18" s="10"/>
+      <c r="CA18" s="10"/>
+      <c r="CB18" s="10"/>
+      <c r="CC18" s="10"/>
+      <c r="CD18" s="10"/>
+      <c r="CE18" s="10"/>
+      <c r="CF18" s="10"/>
+      <c r="CG18" s="10"/>
+      <c r="CH18" s="10"/>
+      <c r="CI18" s="10"/>
+      <c r="CJ18" s="10"/>
+      <c r="CK18" s="10"/>
+      <c r="CL18" s="10"/>
+      <c r="CM18" s="10"/>
+      <c r="CN18" s="10"/>
+      <c r="CO18" s="10"/>
+      <c r="CP18" s="10"/>
+      <c r="CQ18" s="10"/>
+      <c r="CR18" s="10"/>
+      <c r="CS18" s="10"/>
+      <c r="CT18" s="10"/>
+      <c r="CU18" s="10"/>
+      <c r="CV18" s="10"/>
+      <c r="CW18" s="10"/>
+      <c r="CX18" s="10"/>
+      <c r="CY18" s="10"/>
+      <c r="CZ18" s="10"/>
+      <c r="DA18" s="10"/>
+      <c r="DB18" s="10"/>
+      <c r="DC18" s="10"/>
+      <c r="DD18" s="10"/>
+      <c r="DE18" s="10"/>
+      <c r="DF18" s="10"/>
+      <c r="DG18" s="10"/>
+      <c r="DH18" s="10"/>
+      <c r="DI18" s="10"/>
+      <c r="DJ18" s="10"/>
+      <c r="DK18" s="10"/>
+      <c r="DL18" s="10"/>
+      <c r="DM18" s="10"/>
+      <c r="DN18" s="10"/>
+      <c r="DO18" s="10"/>
+      <c r="DP18" s="10"/>
+      <c r="DQ18" s="10"/>
+      <c r="DR18" s="10"/>
+      <c r="DS18" s="10"/>
+      <c r="DT18" s="10"/>
+      <c r="DU18" s="10"/>
+      <c r="DV18" s="10"/>
+      <c r="DW18" s="10"/>
+      <c r="DX18" s="10"/>
+      <c r="DY18" s="10"/>
+      <c r="DZ18" s="10"/>
+      <c r="EA18" s="10"/>
+      <c r="EB18" s="10"/>
+      <c r="EC18" s="10"/>
+      <c r="ED18" s="10"/>
+      <c r="EE18" s="10"/>
+      <c r="EF18" s="10"/>
+      <c r="EG18" s="10"/>
+      <c r="EH18" s="10"/>
+      <c r="EI18" s="10"/>
+      <c r="EJ18" s="10"/>
+      <c r="EK18" s="10"/>
+      <c r="EL18" s="10"/>
+      <c r="EM18" s="10"/>
+      <c r="EN18" s="10"/>
+      <c r="EO18" s="10"/>
+      <c r="EP18" s="10"/>
+      <c r="EQ18" s="10"/>
+      <c r="ER18" s="10"/>
+      <c r="ES18" s="10"/>
+      <c r="ET18" s="10"/>
+      <c r="EU18" s="10"/>
+      <c r="EV18" s="10"/>
+      <c r="EW18" s="10"/>
+      <c r="EX18" s="10"/>
+      <c r="EY18" s="10"/>
+      <c r="EZ18" s="10"/>
+      <c r="FA18" s="10"/>
+      <c r="FB18" s="10"/>
+      <c r="FC18" s="10"/>
+      <c r="FD18" s="10"/>
+      <c r="FE18" s="10"/>
+      <c r="FF18" s="10"/>
+      <c r="FG18" s="10"/>
+      <c r="FH18" s="10"/>
+      <c r="FI18" s="10"/>
+      <c r="FJ18" s="10"/>
+      <c r="FK18" s="10"/>
+      <c r="FL18" s="10"/>
+      <c r="FM18" s="10"/>
+      <c r="FN18" s="10"/>
+      <c r="FO18" s="10"/>
+      <c r="FP18" s="10"/>
+      <c r="FQ18" s="10"/>
+      <c r="FR18" s="10"/>
+      <c r="FS18" s="10"/>
+      <c r="FT18" s="10"/>
+      <c r="FU18" s="10"/>
+      <c r="FV18" s="10"/>
+      <c r="FW18" s="10"/>
+      <c r="FX18" s="10"/>
+      <c r="FY18" s="10"/>
+      <c r="FZ18" s="10"/>
+      <c r="GA18" s="10"/>
+      <c r="GB18" s="10"/>
+      <c r="GC18" s="10"/>
+      <c r="GD18" s="10"/>
+      <c r="GE18" s="10"/>
+      <c r="GF18" s="10"/>
+      <c r="GG18" s="10"/>
+      <c r="GH18" s="10"/>
+      <c r="GI18" s="10"/>
+      <c r="GJ18" s="10"/>
+      <c r="GK18" s="10"/>
+      <c r="GL18" s="10"/>
+      <c r="GM18" s="10"/>
+      <c r="GN18" s="10"/>
+      <c r="GO18" s="10"/>
+      <c r="GP18" s="10"/>
+      <c r="GQ18" s="10"/>
+      <c r="GR18" s="10"/>
+      <c r="GS18" s="10"/>
+      <c r="GT18" s="10"/>
+      <c r="GU18" s="10"/>
+      <c r="GV18" s="10"/>
+      <c r="GW18" s="10"/>
+      <c r="GX18" s="10"/>
+      <c r="GY18" s="10"/>
+      <c r="GZ18" s="10"/>
+      <c r="HA18" s="10"/>
+      <c r="HB18" s="10"/>
+      <c r="HC18" s="10"/>
+      <c r="HD18" s="10"/>
+      <c r="HE18" s="10"/>
+      <c r="HF18" s="10"/>
+      <c r="HG18" s="10"/>
+      <c r="HH18" s="10"/>
+      <c r="HI18" s="10"/>
+      <c r="HJ18" s="10"/>
+      <c r="HK18" s="10"/>
+      <c r="HL18" s="10"/>
+      <c r="HM18" s="10"/>
+      <c r="HN18" s="10"/>
+      <c r="HO18" s="10"/>
+      <c r="HP18" s="10"/>
+      <c r="HQ18" s="10"/>
+      <c r="HR18" s="10"/>
+      <c r="HS18" s="10"/>
+      <c r="HT18" s="10"/>
+      <c r="HU18" s="10"/>
+      <c r="HV18" s="10"/>
+      <c r="HW18" s="10"/>
+      <c r="HX18" s="10"/>
+      <c r="HY18" s="10"/>
+      <c r="HZ18" s="10"/>
+      <c r="IA18" s="10"/>
+      <c r="IB18" s="10"/>
+      <c r="IC18" s="10"/>
+      <c r="ID18" s="10"/>
+      <c r="IE18" s="10"/>
+      <c r="IF18" s="10"/>
+      <c r="IG18" s="10"/>
+      <c r="IH18" s="10"/>
+      <c r="II18" s="10"/>
+      <c r="IJ18" s="10"/>
+      <c r="IK18" s="10"/>
+      <c r="IL18" s="10"/>
+      <c r="IM18" s="10"/>
+      <c r="IN18" s="10"/>
+      <c r="IO18" s="10"/>
+      <c r="IP18" s="10"/>
+      <c r="IQ18" s="10"/>
+      <c r="IR18" s="10"/>
+      <c r="IS18" s="10"/>
+      <c r="IT18" s="10"/>
+      <c r="IU18" s="10"/>
+      <c r="IV18" s="10"/>
+      <c r="IW18" s="10"/>
+      <c r="IX18" s="10"/>
+      <c r="IY18" s="10"/>
+      <c r="IZ18" s="10"/>
+      <c r="JA18" s="10"/>
+      <c r="JB18" s="10"/>
+      <c r="JC18" s="10"/>
+      <c r="JD18" s="10"/>
+      <c r="JE18" s="10"/>
+      <c r="JF18" s="10"/>
+      <c r="JG18" s="10"/>
+      <c r="JH18" s="10"/>
+      <c r="JI18" s="10"/>
+      <c r="JJ18" s="10"/>
+      <c r="JK18" s="10"/>
+      <c r="JL18" s="10"/>
+      <c r="JM18" s="10"/>
+      <c r="JN18" s="10"/>
+    </row>
+    <row r="19" s="6" customFormat="1" ht="28.5">
+      <c r="A19" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="B19" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="29" t="s">
+        <v>154</v>
+      </c>
+      <c r="D19" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="E19" s="29" t="s">
+        <v>156</v>
+      </c>
+      <c r="F19" s="30" t="s">
+        <v>157</v>
+      </c>
+      <c r="G19" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="H19" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="I18" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="J18" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="K18" s="35">
-        <v>2010</v>
-      </c>
-      <c r="L18" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="M18" s="27"/>
-      <c r="N18" s="16"/>
-      <c r="O18" s="36"/>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="36"/>
-      <c r="R18" s="36"/>
-      <c r="S18" s="36"/>
-      <c r="T18" s="36"/>
-      <c r="U18" s="36"/>
-      <c r="V18" s="36"/>
-      <c r="W18" s="36"/>
-      <c r="X18" s="36"/>
-      <c r="Y18" s="36"/>
-      <c r="Z18" s="36"/>
-      <c r="AA18" s="36"/>
-      <c r="AB18" s="36"/>
-      <c r="AC18" s="36"/>
-      <c r="AD18" s="36"/>
-      <c r="AE18" s="36"/>
-      <c r="AF18" s="36"/>
-      <c r="AG18" s="36"/>
-      <c r="AH18" s="36"/>
-      <c r="AI18" s="36"/>
-      <c r="AJ18" s="36"/>
-      <c r="AK18" s="36"/>
-      <c r="AL18" s="36"/>
-      <c r="AM18" s="36"/>
-      <c r="AN18" s="36"/>
-      <c r="AO18" s="36"/>
-      <c r="AP18" s="36"/>
-      <c r="AQ18" s="36"/>
-      <c r="AR18" s="36"/>
-      <c r="AS18" s="36"/>
-      <c r="AT18" s="36"/>
-      <c r="AU18" s="36"/>
-      <c r="AV18" s="36"/>
-      <c r="AW18" s="36"/>
-      <c r="AX18" s="36"/>
-      <c r="AY18" s="36"/>
-      <c r="AZ18" s="36"/>
-      <c r="BA18" s="36"/>
-      <c r="BB18" s="36"/>
-      <c r="BC18" s="36"/>
-      <c r="BD18" s="36"/>
-      <c r="BE18" s="36"/>
-      <c r="BF18" s="36"/>
-      <c r="BG18" s="36"/>
-      <c r="BH18" s="36"/>
-      <c r="BI18" s="36"/>
-      <c r="BJ18" s="36"/>
-      <c r="BK18" s="36"/>
-      <c r="BL18" s="36"/>
-      <c r="BM18" s="36"/>
-      <c r="BN18" s="36"/>
-      <c r="BO18" s="36"/>
-      <c r="BP18" s="36"/>
-      <c r="BQ18" s="36"/>
-      <c r="BR18" s="36"/>
-      <c r="BS18" s="36"/>
-      <c r="BT18" s="36"/>
-      <c r="BU18" s="36"/>
-      <c r="BV18" s="36"/>
-      <c r="BW18" s="36"/>
-      <c r="BX18" s="36"/>
-      <c r="BY18" s="36"/>
-      <c r="BZ18" s="36"/>
-      <c r="CA18" s="36"/>
-      <c r="CB18" s="36"/>
-      <c r="CC18" s="36"/>
-      <c r="CD18" s="36"/>
-      <c r="CE18" s="36"/>
-      <c r="CF18" s="36"/>
-      <c r="CG18" s="36"/>
-      <c r="CH18" s="36"/>
-      <c r="CI18" s="36"/>
-      <c r="CJ18" s="36"/>
-      <c r="CK18" s="36"/>
-      <c r="CL18" s="36"/>
-      <c r="CM18" s="36"/>
-      <c r="CN18" s="36"/>
-      <c r="CO18" s="36"/>
-      <c r="CP18" s="36"/>
-      <c r="CQ18" s="36"/>
-      <c r="CR18" s="36"/>
-      <c r="CS18" s="36"/>
-      <c r="CT18" s="36"/>
-      <c r="CU18" s="36"/>
-      <c r="CV18" s="36"/>
-      <c r="CW18" s="36"/>
-      <c r="CX18" s="36"/>
-      <c r="CY18" s="36"/>
-      <c r="CZ18" s="36"/>
-      <c r="DA18" s="36"/>
-      <c r="DB18" s="36"/>
-      <c r="DC18" s="36"/>
-      <c r="DD18" s="36"/>
-      <c r="DE18" s="36"/>
-      <c r="DF18" s="36"/>
-      <c r="DG18" s="36"/>
-      <c r="DH18" s="36"/>
-      <c r="DI18" s="36"/>
-      <c r="DJ18" s="36"/>
-      <c r="DK18" s="36"/>
-      <c r="DL18" s="36"/>
-      <c r="DM18" s="36"/>
-      <c r="DN18" s="36"/>
-      <c r="DO18" s="36"/>
-      <c r="DP18" s="36"/>
-      <c r="DQ18" s="36"/>
-      <c r="DR18" s="36"/>
-      <c r="DS18" s="36"/>
-      <c r="DT18" s="36"/>
-      <c r="DU18" s="36"/>
-      <c r="DV18" s="36"/>
-      <c r="DW18" s="36"/>
-      <c r="DX18" s="36"/>
-      <c r="DY18" s="36"/>
-      <c r="DZ18" s="36"/>
-      <c r="EA18" s="36"/>
-      <c r="EB18" s="36"/>
-      <c r="EC18" s="36"/>
-      <c r="ED18" s="36"/>
-      <c r="EE18" s="36"/>
-      <c r="EF18" s="36"/>
-      <c r="EG18" s="36"/>
-      <c r="EH18" s="36"/>
-      <c r="EI18" s="36"/>
-      <c r="EJ18" s="36"/>
-      <c r="EK18" s="36"/>
-      <c r="EL18" s="36"/>
-      <c r="EM18" s="36"/>
-      <c r="EN18" s="36"/>
-      <c r="EO18" s="36"/>
-      <c r="EP18" s="36"/>
-      <c r="EQ18" s="36"/>
-      <c r="ER18" s="36"/>
-      <c r="ES18" s="36"/>
-      <c r="ET18" s="36"/>
-      <c r="EU18" s="36"/>
-      <c r="EV18" s="36"/>
-      <c r="EW18" s="36"/>
-      <c r="EX18" s="36"/>
-      <c r="EY18" s="36"/>
-      <c r="EZ18" s="36"/>
-      <c r="FA18" s="36"/>
-      <c r="FB18" s="36"/>
-      <c r="FC18" s="36"/>
-      <c r="FD18" s="36"/>
-      <c r="FE18" s="36"/>
-      <c r="FF18" s="36"/>
-      <c r="FG18" s="36"/>
-      <c r="FH18" s="36"/>
-      <c r="FI18" s="36"/>
-      <c r="FJ18" s="36"/>
-      <c r="FK18" s="36"/>
-      <c r="FL18" s="36"/>
-      <c r="FM18" s="36"/>
-      <c r="FN18" s="36"/>
-      <c r="FO18" s="36"/>
-      <c r="FP18" s="36"/>
-      <c r="FQ18" s="36"/>
-      <c r="FR18" s="36"/>
-      <c r="FS18" s="36"/>
-      <c r="FT18" s="36"/>
-      <c r="FU18" s="36"/>
-      <c r="FV18" s="36"/>
-      <c r="FW18" s="36"/>
-      <c r="FX18" s="36"/>
-      <c r="FY18" s="36"/>
-      <c r="FZ18" s="36"/>
-      <c r="GA18" s="36"/>
-      <c r="GB18" s="36"/>
-      <c r="GC18" s="36"/>
-      <c r="GD18" s="36"/>
-      <c r="GE18" s="36"/>
-      <c r="GF18" s="36"/>
-      <c r="GG18" s="36"/>
-      <c r="GH18" s="36"/>
-      <c r="GI18" s="36"/>
-      <c r="GJ18" s="36"/>
-      <c r="GK18" s="36"/>
-      <c r="GL18" s="36"/>
-      <c r="GM18" s="36"/>
-      <c r="GN18" s="36"/>
-      <c r="GO18" s="36"/>
-      <c r="GP18" s="36"/>
-      <c r="GQ18" s="36"/>
-      <c r="GR18" s="36"/>
-      <c r="GS18" s="36"/>
-      <c r="GT18" s="36"/>
-      <c r="GU18" s="36"/>
-      <c r="GV18" s="36"/>
-      <c r="GW18" s="36"/>
-      <c r="GX18" s="36"/>
-      <c r="GY18" s="36"/>
-      <c r="GZ18" s="36"/>
-      <c r="HA18" s="36"/>
-      <c r="HB18" s="36"/>
-      <c r="HC18" s="36"/>
-      <c r="HD18" s="36"/>
-      <c r="HE18" s="36"/>
-      <c r="HF18" s="36"/>
-      <c r="HG18" s="36"/>
-      <c r="HH18" s="36"/>
-      <c r="HI18" s="36"/>
-      <c r="HJ18" s="36"/>
-      <c r="HK18" s="36"/>
-      <c r="HL18" s="36"/>
-      <c r="HM18" s="36"/>
-      <c r="HN18" s="36"/>
-      <c r="HO18" s="36"/>
-      <c r="HP18" s="36"/>
-      <c r="HQ18" s="36"/>
-      <c r="HR18" s="36"/>
-      <c r="HS18" s="36"/>
-      <c r="HT18" s="36"/>
-      <c r="HU18" s="36"/>
-      <c r="HV18" s="36"/>
-      <c r="HW18" s="36"/>
-      <c r="HX18" s="36"/>
-      <c r="HY18" s="36"/>
-      <c r="HZ18" s="36"/>
-      <c r="IA18" s="36"/>
-      <c r="IB18" s="36"/>
-      <c r="IC18" s="36"/>
-      <c r="ID18" s="36"/>
-      <c r="IE18" s="36"/>
-      <c r="IF18" s="36"/>
-      <c r="IG18" s="36"/>
-      <c r="IH18" s="36"/>
-      <c r="II18" s="36"/>
-      <c r="IJ18" s="36"/>
-      <c r="IK18" s="36"/>
-      <c r="IL18" s="36"/>
-      <c r="IM18" s="36"/>
-      <c r="IN18" s="36"/>
-      <c r="IO18" s="36"/>
-      <c r="IP18" s="36"/>
-      <c r="IQ18" s="36"/>
-      <c r="IR18" s="36"/>
-      <c r="IS18" s="36"/>
-      <c r="IT18" s="36"/>
-      <c r="IU18" s="36"/>
-      <c r="IV18" s="36"/>
-      <c r="IW18" s="36"/>
-      <c r="IX18" s="36"/>
-      <c r="IY18" s="36"/>
-      <c r="IZ18" s="36"/>
-      <c r="JA18" s="36"/>
-      <c r="JB18" s="36"/>
-      <c r="JC18" s="36"/>
-      <c r="JD18" s="36"/>
-      <c r="JE18" s="36"/>
-      <c r="JF18" s="36"/>
-      <c r="JG18" s="36"/>
-      <c r="JH18" s="36"/>
-      <c r="JI18" s="36"/>
-      <c r="JJ18" s="36"/>
-      <c r="JK18" s="36"/>
-      <c r="JL18" s="36"/>
-      <c r="JM18" s="36"/>
-      <c r="JN18" s="36"/>
-    </row>
-    <row r="19" s="6" customFormat="1" ht="25.5">
-      <c r="A19" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="B19" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="C19" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="D19" s="27" t="s">
-        <v>155</v>
-      </c>
-      <c r="E19" s="37" t="s">
-        <v>156</v>
-      </c>
-      <c r="F19" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="G19" s="38"/>
-      <c r="H19" s="27" t="s">
-        <v>84</v>
-      </c>
-      <c r="I19" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="J19" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="K19" s="35">
-        <v>2010</v>
-      </c>
-      <c r="L19" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="M19" s="27"/>
-      <c r="N19" s="16"/>
+      <c r="I19" s="31" t="s">
+        <v>159</v>
+      </c>
+      <c r="J19" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="K19" s="29">
+        <v>2023</v>
+      </c>
+      <c r="L19" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="M19" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="N19" s="30" t="s">
+        <v>162</v>
+      </c>
       <c r="O19" s="10"/>
       <c r="P19" s="10"/>
       <c r="Q19" s="10"/>
@@ -7292,1304 +7322,1304 @@
       <c r="JM19" s="10"/>
       <c r="JN19" s="10"/>
     </row>
-    <row r="20" s="39" customFormat="1" ht="51">
-      <c r="A20" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="B20" s="27" t="s">
+    <row r="20" s="32" customFormat="1" ht="51">
+      <c r="A20" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="B20" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="C20" s="27" t="s">
-        <v>158</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>159</v>
-      </c>
-      <c r="E20" s="27" t="s">
-        <v>160</v>
-      </c>
-      <c r="F20" s="31" t="s">
-        <v>161</v>
-      </c>
-      <c r="G20" s="27" t="s">
-        <v>162</v>
-      </c>
-      <c r="H20" s="27"/>
-      <c r="I20" s="40" t="s">
+      <c r="C20" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="J20" s="41"/>
-      <c r="K20" s="27" t="s">
+      <c r="D20" s="29" t="s">
         <v>164</v>
       </c>
-      <c r="L20" s="27" t="s">
+      <c r="E20" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="F20" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="G20" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="H20" s="29"/>
+      <c r="I20" s="34" t="s">
+        <v>168</v>
+      </c>
+      <c r="J20" s="35"/>
+      <c r="K20" s="29" t="s">
+        <v>169</v>
+      </c>
+      <c r="L20" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="M20" s="27"/>
+      <c r="M20" s="29"/>
       <c r="N20" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="O20" s="42"/>
-      <c r="P20" s="42"/>
-      <c r="Q20" s="42"/>
-      <c r="R20" s="42"/>
-      <c r="S20" s="42"/>
-      <c r="T20" s="42"/>
-      <c r="U20" s="42"/>
-      <c r="V20" s="42"/>
-      <c r="W20" s="42"/>
-      <c r="X20" s="42"/>
-      <c r="Y20" s="42"/>
-      <c r="Z20" s="42"/>
-      <c r="AA20" s="42"/>
-      <c r="AB20" s="42"/>
-      <c r="AC20" s="42"/>
-      <c r="AD20" s="42"/>
-      <c r="AE20" s="42"/>
-      <c r="AF20" s="42"/>
-      <c r="AG20" s="42"/>
-      <c r="AH20" s="42"/>
-      <c r="AI20" s="42"/>
-      <c r="AJ20" s="42"/>
-      <c r="AK20" s="42"/>
-      <c r="AL20" s="42"/>
-      <c r="AM20" s="42"/>
-      <c r="AN20" s="42"/>
-      <c r="AO20" s="42"/>
-      <c r="AP20" s="42"/>
-      <c r="AQ20" s="42"/>
-      <c r="AR20" s="42"/>
-      <c r="AS20" s="42"/>
-      <c r="AT20" s="42"/>
-      <c r="AU20" s="42"/>
-      <c r="AV20" s="42"/>
-      <c r="AW20" s="42"/>
-      <c r="AX20" s="42"/>
-      <c r="AY20" s="42"/>
-      <c r="AZ20" s="42"/>
-      <c r="BA20" s="42"/>
-      <c r="BB20" s="42"/>
-      <c r="BC20" s="42"/>
-      <c r="BD20" s="42"/>
-      <c r="BE20" s="42"/>
-      <c r="BF20" s="42"/>
-      <c r="BG20" s="42"/>
-      <c r="BH20" s="42"/>
-      <c r="BI20" s="42"/>
-      <c r="BJ20" s="42"/>
-      <c r="BK20" s="42"/>
-      <c r="BL20" s="42"/>
-      <c r="BM20" s="42"/>
-      <c r="BN20" s="42"/>
-      <c r="BO20" s="42"/>
-      <c r="BP20" s="42"/>
-      <c r="BQ20" s="42"/>
-      <c r="BR20" s="42"/>
-      <c r="BS20" s="42"/>
-      <c r="BT20" s="42"/>
-      <c r="BU20" s="42"/>
-      <c r="BV20" s="42"/>
-      <c r="BW20" s="42"/>
-      <c r="BX20" s="42"/>
-      <c r="BY20" s="42"/>
-      <c r="BZ20" s="42"/>
-      <c r="CA20" s="42"/>
-      <c r="CB20" s="42"/>
-      <c r="CC20" s="42"/>
-      <c r="CD20" s="42"/>
-      <c r="CE20" s="42"/>
-      <c r="CF20" s="42"/>
-      <c r="CG20" s="42"/>
-      <c r="CH20" s="42"/>
-      <c r="CI20" s="42"/>
-      <c r="CJ20" s="42"/>
-      <c r="CK20" s="42"/>
-      <c r="CL20" s="42"/>
-      <c r="CM20" s="42"/>
-      <c r="CN20" s="42"/>
-      <c r="CO20" s="42"/>
-      <c r="CP20" s="42"/>
-      <c r="CQ20" s="42"/>
-      <c r="CR20" s="42"/>
-      <c r="CS20" s="42"/>
-      <c r="CT20" s="42"/>
-      <c r="CU20" s="42"/>
-      <c r="CV20" s="42"/>
-      <c r="CW20" s="42"/>
-      <c r="CX20" s="42"/>
-      <c r="CY20" s="42"/>
-      <c r="CZ20" s="42"/>
-      <c r="DA20" s="42"/>
-      <c r="DB20" s="42"/>
-      <c r="DC20" s="42"/>
-      <c r="DD20" s="42"/>
-      <c r="DE20" s="42"/>
-      <c r="DF20" s="42"/>
-      <c r="DG20" s="42"/>
-      <c r="DH20" s="42"/>
-      <c r="DI20" s="42"/>
-      <c r="DJ20" s="42"/>
-      <c r="DK20" s="42"/>
-      <c r="DL20" s="42"/>
-      <c r="DM20" s="42"/>
-      <c r="DN20" s="42"/>
-      <c r="DO20" s="42"/>
-      <c r="DP20" s="42"/>
-      <c r="DQ20" s="42"/>
-      <c r="DR20" s="42"/>
-      <c r="DS20" s="42"/>
-      <c r="DT20" s="42"/>
-      <c r="DU20" s="42"/>
-      <c r="DV20" s="42"/>
-      <c r="DW20" s="42"/>
-      <c r="DX20" s="42"/>
-      <c r="DY20" s="42"/>
-      <c r="DZ20" s="42"/>
-      <c r="EA20" s="42"/>
-      <c r="EB20" s="42"/>
-      <c r="EC20" s="42"/>
-      <c r="ED20" s="42"/>
-      <c r="EE20" s="42"/>
-      <c r="EF20" s="42"/>
-      <c r="EG20" s="42"/>
-      <c r="EH20" s="42"/>
-      <c r="EI20" s="42"/>
-      <c r="EJ20" s="42"/>
-      <c r="EK20" s="42"/>
-      <c r="EL20" s="42"/>
-      <c r="EM20" s="42"/>
-      <c r="EN20" s="42"/>
-      <c r="EO20" s="42"/>
-      <c r="EP20" s="42"/>
-      <c r="EQ20" s="42"/>
-      <c r="ER20" s="42"/>
-      <c r="ES20" s="42"/>
-      <c r="ET20" s="42"/>
-      <c r="EU20" s="42"/>
-      <c r="EV20" s="42"/>
-      <c r="EW20" s="42"/>
-      <c r="EX20" s="42"/>
-      <c r="EY20" s="42"/>
-      <c r="EZ20" s="42"/>
-      <c r="FA20" s="42"/>
-      <c r="FB20" s="42"/>
-      <c r="FC20" s="42"/>
-      <c r="FD20" s="42"/>
-      <c r="FE20" s="42"/>
-      <c r="FF20" s="42"/>
-      <c r="FG20" s="42"/>
-      <c r="FH20" s="42"/>
-      <c r="FI20" s="42"/>
-      <c r="FJ20" s="42"/>
-      <c r="FK20" s="42"/>
-      <c r="FL20" s="42"/>
-      <c r="FM20" s="42"/>
-      <c r="FN20" s="42"/>
-      <c r="FO20" s="42"/>
-      <c r="FP20" s="42"/>
-      <c r="FQ20" s="42"/>
-      <c r="FR20" s="42"/>
-      <c r="FS20" s="42"/>
-      <c r="FT20" s="42"/>
-      <c r="FU20" s="42"/>
-      <c r="FV20" s="42"/>
-      <c r="FW20" s="42"/>
-      <c r="FX20" s="42"/>
-      <c r="FY20" s="42"/>
-      <c r="FZ20" s="42"/>
-      <c r="GA20" s="42"/>
-      <c r="GB20" s="42"/>
-      <c r="GC20" s="42"/>
-      <c r="GD20" s="42"/>
-      <c r="GE20" s="42"/>
-      <c r="GF20" s="42"/>
-      <c r="GG20" s="42"/>
-      <c r="GH20" s="42"/>
-      <c r="GI20" s="42"/>
-      <c r="GJ20" s="42"/>
-      <c r="GK20" s="42"/>
-      <c r="GL20" s="42"/>
-      <c r="GM20" s="42"/>
-      <c r="GN20" s="42"/>
-      <c r="GO20" s="42"/>
-      <c r="GP20" s="42"/>
-      <c r="GQ20" s="42"/>
-      <c r="GR20" s="42"/>
-      <c r="GS20" s="42"/>
-      <c r="GT20" s="42"/>
-      <c r="GU20" s="42"/>
-      <c r="GV20" s="42"/>
-      <c r="GW20" s="42"/>
-      <c r="GX20" s="42"/>
-      <c r="GY20" s="42"/>
-      <c r="GZ20" s="42"/>
-      <c r="HA20" s="42"/>
-      <c r="HB20" s="42"/>
-      <c r="HC20" s="42"/>
-      <c r="HD20" s="42"/>
-      <c r="HE20" s="42"/>
-      <c r="HF20" s="42"/>
-      <c r="HG20" s="42"/>
-      <c r="HH20" s="42"/>
-      <c r="HI20" s="42"/>
-      <c r="HJ20" s="42"/>
-      <c r="HK20" s="42"/>
-      <c r="HL20" s="42"/>
-      <c r="HM20" s="42"/>
-      <c r="HN20" s="42"/>
-      <c r="HO20" s="42"/>
-      <c r="HP20" s="42"/>
-      <c r="HQ20" s="42"/>
-      <c r="HR20" s="42"/>
-      <c r="HS20" s="42"/>
-      <c r="HT20" s="42"/>
-      <c r="HU20" s="42"/>
-      <c r="HV20" s="42"/>
-      <c r="HW20" s="42"/>
-      <c r="HX20" s="42"/>
-      <c r="HY20" s="42"/>
-      <c r="HZ20" s="42"/>
-      <c r="IA20" s="42"/>
-      <c r="IB20" s="42"/>
-      <c r="IC20" s="42"/>
-      <c r="ID20" s="42"/>
-      <c r="IE20" s="42"/>
-      <c r="IF20" s="42"/>
-      <c r="IG20" s="42"/>
-      <c r="IH20" s="42"/>
-      <c r="II20" s="42"/>
-      <c r="IJ20" s="42"/>
-      <c r="IK20" s="42"/>
-      <c r="IL20" s="42"/>
-      <c r="IM20" s="42"/>
-      <c r="IN20" s="42"/>
-      <c r="IO20" s="42"/>
-      <c r="IP20" s="42"/>
-      <c r="IQ20" s="42"/>
-      <c r="IR20" s="42"/>
-      <c r="IS20" s="42"/>
-      <c r="IT20" s="42"/>
-      <c r="IU20" s="42"/>
-      <c r="IV20" s="42"/>
-      <c r="IW20" s="42"/>
-      <c r="IX20" s="42"/>
-      <c r="IY20" s="42"/>
-      <c r="IZ20" s="42"/>
-      <c r="JA20" s="42"/>
-      <c r="JB20" s="42"/>
-      <c r="JC20" s="42"/>
-      <c r="JD20" s="42"/>
-      <c r="JE20" s="42"/>
-      <c r="JF20" s="42"/>
-      <c r="JG20" s="42"/>
-      <c r="JH20" s="42"/>
-      <c r="JI20" s="42"/>
-      <c r="JJ20" s="42"/>
-      <c r="JK20" s="42"/>
-      <c r="JL20" s="42"/>
-      <c r="JM20" s="42"/>
-      <c r="JN20" s="42"/>
+        <v>170</v>
+      </c>
+      <c r="O20" s="36"/>
+      <c r="P20" s="36"/>
+      <c r="Q20" s="36"/>
+      <c r="R20" s="36"/>
+      <c r="S20" s="36"/>
+      <c r="T20" s="36"/>
+      <c r="U20" s="36"/>
+      <c r="V20" s="36"/>
+      <c r="W20" s="36"/>
+      <c r="X20" s="36"/>
+      <c r="Y20" s="36"/>
+      <c r="Z20" s="36"/>
+      <c r="AA20" s="36"/>
+      <c r="AB20" s="36"/>
+      <c r="AC20" s="36"/>
+      <c r="AD20" s="36"/>
+      <c r="AE20" s="36"/>
+      <c r="AF20" s="36"/>
+      <c r="AG20" s="36"/>
+      <c r="AH20" s="36"/>
+      <c r="AI20" s="36"/>
+      <c r="AJ20" s="36"/>
+      <c r="AK20" s="36"/>
+      <c r="AL20" s="36"/>
+      <c r="AM20" s="36"/>
+      <c r="AN20" s="36"/>
+      <c r="AO20" s="36"/>
+      <c r="AP20" s="36"/>
+      <c r="AQ20" s="36"/>
+      <c r="AR20" s="36"/>
+      <c r="AS20" s="36"/>
+      <c r="AT20" s="36"/>
+      <c r="AU20" s="36"/>
+      <c r="AV20" s="36"/>
+      <c r="AW20" s="36"/>
+      <c r="AX20" s="36"/>
+      <c r="AY20" s="36"/>
+      <c r="AZ20" s="36"/>
+      <c r="BA20" s="36"/>
+      <c r="BB20" s="36"/>
+      <c r="BC20" s="36"/>
+      <c r="BD20" s="36"/>
+      <c r="BE20" s="36"/>
+      <c r="BF20" s="36"/>
+      <c r="BG20" s="36"/>
+      <c r="BH20" s="36"/>
+      <c r="BI20" s="36"/>
+      <c r="BJ20" s="36"/>
+      <c r="BK20" s="36"/>
+      <c r="BL20" s="36"/>
+      <c r="BM20" s="36"/>
+      <c r="BN20" s="36"/>
+      <c r="BO20" s="36"/>
+      <c r="BP20" s="36"/>
+      <c r="BQ20" s="36"/>
+      <c r="BR20" s="36"/>
+      <c r="BS20" s="36"/>
+      <c r="BT20" s="36"/>
+      <c r="BU20" s="36"/>
+      <c r="BV20" s="36"/>
+      <c r="BW20" s="36"/>
+      <c r="BX20" s="36"/>
+      <c r="BY20" s="36"/>
+      <c r="BZ20" s="36"/>
+      <c r="CA20" s="36"/>
+      <c r="CB20" s="36"/>
+      <c r="CC20" s="36"/>
+      <c r="CD20" s="36"/>
+      <c r="CE20" s="36"/>
+      <c r="CF20" s="36"/>
+      <c r="CG20" s="36"/>
+      <c r="CH20" s="36"/>
+      <c r="CI20" s="36"/>
+      <c r="CJ20" s="36"/>
+      <c r="CK20" s="36"/>
+      <c r="CL20" s="36"/>
+      <c r="CM20" s="36"/>
+      <c r="CN20" s="36"/>
+      <c r="CO20" s="36"/>
+      <c r="CP20" s="36"/>
+      <c r="CQ20" s="36"/>
+      <c r="CR20" s="36"/>
+      <c r="CS20" s="36"/>
+      <c r="CT20" s="36"/>
+      <c r="CU20" s="36"/>
+      <c r="CV20" s="36"/>
+      <c r="CW20" s="36"/>
+      <c r="CX20" s="36"/>
+      <c r="CY20" s="36"/>
+      <c r="CZ20" s="36"/>
+      <c r="DA20" s="36"/>
+      <c r="DB20" s="36"/>
+      <c r="DC20" s="36"/>
+      <c r="DD20" s="36"/>
+      <c r="DE20" s="36"/>
+      <c r="DF20" s="36"/>
+      <c r="DG20" s="36"/>
+      <c r="DH20" s="36"/>
+      <c r="DI20" s="36"/>
+      <c r="DJ20" s="36"/>
+      <c r="DK20" s="36"/>
+      <c r="DL20" s="36"/>
+      <c r="DM20" s="36"/>
+      <c r="DN20" s="36"/>
+      <c r="DO20" s="36"/>
+      <c r="DP20" s="36"/>
+      <c r="DQ20" s="36"/>
+      <c r="DR20" s="36"/>
+      <c r="DS20" s="36"/>
+      <c r="DT20" s="36"/>
+      <c r="DU20" s="36"/>
+      <c r="DV20" s="36"/>
+      <c r="DW20" s="36"/>
+      <c r="DX20" s="36"/>
+      <c r="DY20" s="36"/>
+      <c r="DZ20" s="36"/>
+      <c r="EA20" s="36"/>
+      <c r="EB20" s="36"/>
+      <c r="EC20" s="36"/>
+      <c r="ED20" s="36"/>
+      <c r="EE20" s="36"/>
+      <c r="EF20" s="36"/>
+      <c r="EG20" s="36"/>
+      <c r="EH20" s="36"/>
+      <c r="EI20" s="36"/>
+      <c r="EJ20" s="36"/>
+      <c r="EK20" s="36"/>
+      <c r="EL20" s="36"/>
+      <c r="EM20" s="36"/>
+      <c r="EN20" s="36"/>
+      <c r="EO20" s="36"/>
+      <c r="EP20" s="36"/>
+      <c r="EQ20" s="36"/>
+      <c r="ER20" s="36"/>
+      <c r="ES20" s="36"/>
+      <c r="ET20" s="36"/>
+      <c r="EU20" s="36"/>
+      <c r="EV20" s="36"/>
+      <c r="EW20" s="36"/>
+      <c r="EX20" s="36"/>
+      <c r="EY20" s="36"/>
+      <c r="EZ20" s="36"/>
+      <c r="FA20" s="36"/>
+      <c r="FB20" s="36"/>
+      <c r="FC20" s="36"/>
+      <c r="FD20" s="36"/>
+      <c r="FE20" s="36"/>
+      <c r="FF20" s="36"/>
+      <c r="FG20" s="36"/>
+      <c r="FH20" s="36"/>
+      <c r="FI20" s="36"/>
+      <c r="FJ20" s="36"/>
+      <c r="FK20" s="36"/>
+      <c r="FL20" s="36"/>
+      <c r="FM20" s="36"/>
+      <c r="FN20" s="36"/>
+      <c r="FO20" s="36"/>
+      <c r="FP20" s="36"/>
+      <c r="FQ20" s="36"/>
+      <c r="FR20" s="36"/>
+      <c r="FS20" s="36"/>
+      <c r="FT20" s="36"/>
+      <c r="FU20" s="36"/>
+      <c r="FV20" s="36"/>
+      <c r="FW20" s="36"/>
+      <c r="FX20" s="36"/>
+      <c r="FY20" s="36"/>
+      <c r="FZ20" s="36"/>
+      <c r="GA20" s="36"/>
+      <c r="GB20" s="36"/>
+      <c r="GC20" s="36"/>
+      <c r="GD20" s="36"/>
+      <c r="GE20" s="36"/>
+      <c r="GF20" s="36"/>
+      <c r="GG20" s="36"/>
+      <c r="GH20" s="36"/>
+      <c r="GI20" s="36"/>
+      <c r="GJ20" s="36"/>
+      <c r="GK20" s="36"/>
+      <c r="GL20" s="36"/>
+      <c r="GM20" s="36"/>
+      <c r="GN20" s="36"/>
+      <c r="GO20" s="36"/>
+      <c r="GP20" s="36"/>
+      <c r="GQ20" s="36"/>
+      <c r="GR20" s="36"/>
+      <c r="GS20" s="36"/>
+      <c r="GT20" s="36"/>
+      <c r="GU20" s="36"/>
+      <c r="GV20" s="36"/>
+      <c r="GW20" s="36"/>
+      <c r="GX20" s="36"/>
+      <c r="GY20" s="36"/>
+      <c r="GZ20" s="36"/>
+      <c r="HA20" s="36"/>
+      <c r="HB20" s="36"/>
+      <c r="HC20" s="36"/>
+      <c r="HD20" s="36"/>
+      <c r="HE20" s="36"/>
+      <c r="HF20" s="36"/>
+      <c r="HG20" s="36"/>
+      <c r="HH20" s="36"/>
+      <c r="HI20" s="36"/>
+      <c r="HJ20" s="36"/>
+      <c r="HK20" s="36"/>
+      <c r="HL20" s="36"/>
+      <c r="HM20" s="36"/>
+      <c r="HN20" s="36"/>
+      <c r="HO20" s="36"/>
+      <c r="HP20" s="36"/>
+      <c r="HQ20" s="36"/>
+      <c r="HR20" s="36"/>
+      <c r="HS20" s="36"/>
+      <c r="HT20" s="36"/>
+      <c r="HU20" s="36"/>
+      <c r="HV20" s="36"/>
+      <c r="HW20" s="36"/>
+      <c r="HX20" s="36"/>
+      <c r="HY20" s="36"/>
+      <c r="HZ20" s="36"/>
+      <c r="IA20" s="36"/>
+      <c r="IB20" s="36"/>
+      <c r="IC20" s="36"/>
+      <c r="ID20" s="36"/>
+      <c r="IE20" s="36"/>
+      <c r="IF20" s="36"/>
+      <c r="IG20" s="36"/>
+      <c r="IH20" s="36"/>
+      <c r="II20" s="36"/>
+      <c r="IJ20" s="36"/>
+      <c r="IK20" s="36"/>
+      <c r="IL20" s="36"/>
+      <c r="IM20" s="36"/>
+      <c r="IN20" s="36"/>
+      <c r="IO20" s="36"/>
+      <c r="IP20" s="36"/>
+      <c r="IQ20" s="36"/>
+      <c r="IR20" s="36"/>
+      <c r="IS20" s="36"/>
+      <c r="IT20" s="36"/>
+      <c r="IU20" s="36"/>
+      <c r="IV20" s="36"/>
+      <c r="IW20" s="36"/>
+      <c r="IX20" s="36"/>
+      <c r="IY20" s="36"/>
+      <c r="IZ20" s="36"/>
+      <c r="JA20" s="36"/>
+      <c r="JB20" s="36"/>
+      <c r="JC20" s="36"/>
+      <c r="JD20" s="36"/>
+      <c r="JE20" s="36"/>
+      <c r="JF20" s="36"/>
+      <c r="JG20" s="36"/>
+      <c r="JH20" s="36"/>
+      <c r="JI20" s="36"/>
+      <c r="JJ20" s="36"/>
+      <c r="JK20" s="36"/>
+      <c r="JL20" s="36"/>
+      <c r="JM20" s="36"/>
+      <c r="JN20" s="36"/>
     </row>
-    <row r="21" s="43" customFormat="1" ht="25.5">
-      <c r="A21" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="B21" s="27" t="s">
+    <row r="21" s="37" customFormat="1" ht="25.5">
+      <c r="A21" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="B21" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="C21" s="27" t="s">
-        <v>158</v>
-      </c>
-      <c r="D21" s="27" t="s">
-        <v>166</v>
-      </c>
-      <c r="E21" s="27" t="s">
-        <v>167</v>
-      </c>
-      <c r="F21" s="31" t="s">
-        <v>168</v>
-      </c>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="I21" s="32" t="s">
-        <v>170</v>
-      </c>
-      <c r="J21" s="41"/>
-      <c r="K21" s="27">
+      <c r="C21" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="D21" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="E21" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="F21" s="33" t="s">
+        <v>173</v>
+      </c>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29" t="s">
+        <v>174</v>
+      </c>
+      <c r="I21" s="38" t="s">
+        <v>175</v>
+      </c>
+      <c r="J21" s="35"/>
+      <c r="K21" s="29">
         <v>2025</v>
       </c>
-      <c r="L21" s="27" t="s">
-        <v>171</v>
-      </c>
-      <c r="M21" s="27"/>
+      <c r="L21" s="29" t="s">
+        <v>176</v>
+      </c>
+      <c r="M21" s="29"/>
       <c r="N21" s="16"/>
-      <c r="O21" s="43"/>
-      <c r="P21" s="43"/>
-      <c r="Q21" s="43"/>
-      <c r="R21" s="43"/>
-      <c r="S21" s="43"/>
-      <c r="T21" s="43"/>
-      <c r="U21" s="43"/>
-      <c r="V21" s="43"/>
-      <c r="W21" s="43"/>
-      <c r="X21" s="43"/>
-      <c r="Y21" s="43"/>
-      <c r="Z21" s="43"/>
-      <c r="AA21" s="43"/>
-      <c r="AB21" s="43"/>
-      <c r="AC21" s="43"/>
-      <c r="AD21" s="43"/>
-      <c r="AE21" s="43"/>
-      <c r="AF21" s="43"/>
-      <c r="AG21" s="43"/>
-      <c r="AH21" s="43"/>
-      <c r="AI21" s="43"/>
-      <c r="AJ21" s="43"/>
-      <c r="AK21" s="43"/>
-      <c r="AL21" s="43"/>
-      <c r="AM21" s="43"/>
-      <c r="AN21" s="43"/>
-      <c r="AO21" s="43"/>
-      <c r="AP21" s="43"/>
-      <c r="AQ21" s="43"/>
-      <c r="AR21" s="43"/>
-      <c r="AS21" s="43"/>
-      <c r="AT21" s="43"/>
-      <c r="AU21" s="43"/>
-      <c r="AV21" s="43"/>
-      <c r="AW21" s="43"/>
-      <c r="AX21" s="43"/>
-      <c r="AY21" s="43"/>
-      <c r="AZ21" s="43"/>
-      <c r="BA21" s="43"/>
-      <c r="BB21" s="43"/>
-      <c r="BC21" s="43"/>
-      <c r="BD21" s="43"/>
-      <c r="BE21" s="43"/>
-      <c r="BF21" s="43"/>
-      <c r="BG21" s="43"/>
-      <c r="BH21" s="43"/>
-      <c r="BI21" s="43"/>
-      <c r="BJ21" s="43"/>
-      <c r="BK21" s="43"/>
-      <c r="BL21" s="43"/>
-      <c r="BM21" s="43"/>
-      <c r="BN21" s="43"/>
-      <c r="BO21" s="43"/>
-      <c r="BP21" s="43"/>
-      <c r="BQ21" s="43"/>
-      <c r="BR21" s="43"/>
-      <c r="BS21" s="43"/>
-      <c r="BT21" s="43"/>
-      <c r="BU21" s="43"/>
-      <c r="BV21" s="43"/>
-      <c r="BW21" s="43"/>
-      <c r="BX21" s="43"/>
-      <c r="BY21" s="43"/>
-      <c r="BZ21" s="43"/>
-      <c r="CA21" s="43"/>
-      <c r="CB21" s="43"/>
-      <c r="CC21" s="43"/>
-      <c r="CD21" s="43"/>
-      <c r="CE21" s="43"/>
-      <c r="CF21" s="43"/>
-      <c r="CG21" s="43"/>
-      <c r="CH21" s="43"/>
-      <c r="CI21" s="43"/>
-      <c r="CJ21" s="43"/>
-      <c r="CK21" s="43"/>
-      <c r="CL21" s="43"/>
-      <c r="CM21" s="43"/>
-      <c r="CN21" s="43"/>
-      <c r="CO21" s="43"/>
-      <c r="CP21" s="43"/>
-      <c r="CQ21" s="43"/>
-      <c r="CR21" s="43"/>
-      <c r="CS21" s="43"/>
-      <c r="CT21" s="43"/>
-      <c r="CU21" s="43"/>
-      <c r="CV21" s="43"/>
-      <c r="CW21" s="43"/>
-      <c r="CX21" s="43"/>
-      <c r="CY21" s="43"/>
-      <c r="CZ21" s="43"/>
-      <c r="DA21" s="43"/>
-      <c r="DB21" s="43"/>
-      <c r="DC21" s="43"/>
-      <c r="DD21" s="43"/>
-      <c r="DE21" s="43"/>
-      <c r="DF21" s="43"/>
-      <c r="DG21" s="43"/>
-      <c r="DH21" s="43"/>
-      <c r="DI21" s="43"/>
-      <c r="DJ21" s="43"/>
-      <c r="DK21" s="43"/>
-      <c r="DL21" s="43"/>
-      <c r="DM21" s="43"/>
-      <c r="DN21" s="43"/>
-      <c r="DO21" s="43"/>
-      <c r="DP21" s="43"/>
-      <c r="DQ21" s="43"/>
-      <c r="DR21" s="43"/>
-      <c r="DS21" s="43"/>
-      <c r="DT21" s="43"/>
-      <c r="DU21" s="43"/>
-      <c r="DV21" s="43"/>
-      <c r="DW21" s="43"/>
-      <c r="DX21" s="43"/>
-      <c r="DY21" s="43"/>
-      <c r="DZ21" s="43"/>
-      <c r="EA21" s="43"/>
-      <c r="EB21" s="43"/>
-      <c r="EC21" s="43"/>
-      <c r="ED21" s="43"/>
-      <c r="EE21" s="43"/>
-      <c r="EF21" s="43"/>
-      <c r="EG21" s="43"/>
-      <c r="EH21" s="43"/>
-      <c r="EI21" s="43"/>
-      <c r="EJ21" s="43"/>
-      <c r="EK21" s="43"/>
-      <c r="EL21" s="43"/>
-      <c r="EM21" s="43"/>
-      <c r="EN21" s="43"/>
-      <c r="EO21" s="43"/>
-      <c r="EP21" s="43"/>
-      <c r="EQ21" s="43"/>
-      <c r="ER21" s="43"/>
-      <c r="ES21" s="43"/>
-      <c r="ET21" s="43"/>
-      <c r="EU21" s="43"/>
-      <c r="EV21" s="43"/>
-      <c r="EW21" s="43"/>
-      <c r="EX21" s="43"/>
-      <c r="EY21" s="43"/>
-      <c r="EZ21" s="43"/>
-      <c r="FA21" s="43"/>
-      <c r="FB21" s="43"/>
-      <c r="FC21" s="43"/>
-      <c r="FD21" s="43"/>
-      <c r="FE21" s="43"/>
-      <c r="FF21" s="43"/>
-      <c r="FG21" s="43"/>
-      <c r="FH21" s="43"/>
-      <c r="FI21" s="43"/>
-      <c r="FJ21" s="43"/>
-      <c r="FK21" s="43"/>
-      <c r="FL21" s="43"/>
-      <c r="FM21" s="43"/>
-      <c r="FN21" s="43"/>
-      <c r="FO21" s="43"/>
-      <c r="FP21" s="43"/>
-      <c r="FQ21" s="43"/>
-      <c r="FR21" s="43"/>
-      <c r="FS21" s="43"/>
-      <c r="FT21" s="43"/>
-      <c r="FU21" s="43"/>
-      <c r="FV21" s="43"/>
-      <c r="FW21" s="43"/>
-      <c r="FX21" s="43"/>
-      <c r="FY21" s="43"/>
-      <c r="FZ21" s="43"/>
-      <c r="GA21" s="43"/>
-      <c r="GB21" s="43"/>
-      <c r="GC21" s="43"/>
-      <c r="GD21" s="43"/>
-      <c r="GE21" s="43"/>
-      <c r="GF21" s="43"/>
-      <c r="GG21" s="43"/>
-      <c r="GH21" s="43"/>
-      <c r="GI21" s="43"/>
-      <c r="GJ21" s="43"/>
-      <c r="GK21" s="43"/>
-      <c r="GL21" s="43"/>
-      <c r="GM21" s="43"/>
-      <c r="GN21" s="43"/>
-      <c r="GO21" s="43"/>
-      <c r="GP21" s="43"/>
-      <c r="GQ21" s="43"/>
-      <c r="GR21" s="43"/>
-      <c r="GS21" s="43"/>
-      <c r="GT21" s="43"/>
-      <c r="GU21" s="43"/>
-      <c r="GV21" s="43"/>
-      <c r="GW21" s="43"/>
-      <c r="GX21" s="43"/>
-      <c r="GY21" s="43"/>
-      <c r="GZ21" s="43"/>
-      <c r="HA21" s="43"/>
-      <c r="HB21" s="43"/>
-      <c r="HC21" s="43"/>
-      <c r="HD21" s="43"/>
-      <c r="HE21" s="43"/>
-      <c r="HF21" s="43"/>
-      <c r="HG21" s="43"/>
-      <c r="HH21" s="43"/>
-      <c r="HI21" s="43"/>
-      <c r="HJ21" s="43"/>
-      <c r="HK21" s="43"/>
-      <c r="HL21" s="43"/>
-      <c r="HM21" s="43"/>
-      <c r="HN21" s="43"/>
-      <c r="HO21" s="43"/>
-      <c r="HP21" s="43"/>
-      <c r="HQ21" s="43"/>
-      <c r="HR21" s="43"/>
-      <c r="HS21" s="43"/>
-      <c r="HT21" s="43"/>
-      <c r="HU21" s="43"/>
-      <c r="HV21" s="43"/>
-      <c r="HW21" s="43"/>
-      <c r="HX21" s="43"/>
-      <c r="HY21" s="43"/>
-      <c r="HZ21" s="43"/>
-      <c r="IA21" s="43"/>
-      <c r="IB21" s="43"/>
-      <c r="IC21" s="43"/>
-      <c r="ID21" s="43"/>
-      <c r="IE21" s="43"/>
-      <c r="IF21" s="43"/>
-      <c r="IG21" s="43"/>
-      <c r="IH21" s="43"/>
-      <c r="II21" s="43"/>
-      <c r="IJ21" s="43"/>
-      <c r="IK21" s="43"/>
-      <c r="IL21" s="43"/>
-      <c r="IM21" s="43"/>
-      <c r="IN21" s="43"/>
-      <c r="IO21" s="43"/>
-      <c r="IP21" s="43"/>
-      <c r="IQ21" s="43"/>
-      <c r="IR21" s="43"/>
-      <c r="IS21" s="43"/>
-      <c r="IT21" s="43"/>
-      <c r="IU21" s="43"/>
-      <c r="IV21" s="43"/>
-      <c r="IW21" s="43"/>
-      <c r="IX21" s="43"/>
-      <c r="IY21" s="43"/>
-      <c r="IZ21" s="43"/>
-      <c r="JA21" s="43"/>
-      <c r="JB21" s="43"/>
-      <c r="JC21" s="43"/>
-      <c r="JD21" s="43"/>
-      <c r="JE21" s="43"/>
-      <c r="JF21" s="43"/>
-      <c r="JG21" s="43"/>
-      <c r="JH21" s="43"/>
-      <c r="JI21" s="43"/>
-      <c r="JJ21" s="43"/>
-      <c r="JK21" s="43"/>
-      <c r="JL21" s="43"/>
-      <c r="JM21" s="43"/>
-      <c r="JN21" s="43"/>
+      <c r="O21" s="37"/>
+      <c r="P21" s="37"/>
+      <c r="Q21" s="37"/>
+      <c r="R21" s="37"/>
+      <c r="S21" s="37"/>
+      <c r="T21" s="37"/>
+      <c r="U21" s="37"/>
+      <c r="V21" s="37"/>
+      <c r="W21" s="37"/>
+      <c r="X21" s="37"/>
+      <c r="Y21" s="37"/>
+      <c r="Z21" s="37"/>
+      <c r="AA21" s="37"/>
+      <c r="AB21" s="37"/>
+      <c r="AC21" s="37"/>
+      <c r="AD21" s="37"/>
+      <c r="AE21" s="37"/>
+      <c r="AF21" s="37"/>
+      <c r="AG21" s="37"/>
+      <c r="AH21" s="37"/>
+      <c r="AI21" s="37"/>
+      <c r="AJ21" s="37"/>
+      <c r="AK21" s="37"/>
+      <c r="AL21" s="37"/>
+      <c r="AM21" s="37"/>
+      <c r="AN21" s="37"/>
+      <c r="AO21" s="37"/>
+      <c r="AP21" s="37"/>
+      <c r="AQ21" s="37"/>
+      <c r="AR21" s="37"/>
+      <c r="AS21" s="37"/>
+      <c r="AT21" s="37"/>
+      <c r="AU21" s="37"/>
+      <c r="AV21" s="37"/>
+      <c r="AW21" s="37"/>
+      <c r="AX21" s="37"/>
+      <c r="AY21" s="37"/>
+      <c r="AZ21" s="37"/>
+      <c r="BA21" s="37"/>
+      <c r="BB21" s="37"/>
+      <c r="BC21" s="37"/>
+      <c r="BD21" s="37"/>
+      <c r="BE21" s="37"/>
+      <c r="BF21" s="37"/>
+      <c r="BG21" s="37"/>
+      <c r="BH21" s="37"/>
+      <c r="BI21" s="37"/>
+      <c r="BJ21" s="37"/>
+      <c r="BK21" s="37"/>
+      <c r="BL21" s="37"/>
+      <c r="BM21" s="37"/>
+      <c r="BN21" s="37"/>
+      <c r="BO21" s="37"/>
+      <c r="BP21" s="37"/>
+      <c r="BQ21" s="37"/>
+      <c r="BR21" s="37"/>
+      <c r="BS21" s="37"/>
+      <c r="BT21" s="37"/>
+      <c r="BU21" s="37"/>
+      <c r="BV21" s="37"/>
+      <c r="BW21" s="37"/>
+      <c r="BX21" s="37"/>
+      <c r="BY21" s="37"/>
+      <c r="BZ21" s="37"/>
+      <c r="CA21" s="37"/>
+      <c r="CB21" s="37"/>
+      <c r="CC21" s="37"/>
+      <c r="CD21" s="37"/>
+      <c r="CE21" s="37"/>
+      <c r="CF21" s="37"/>
+      <c r="CG21" s="37"/>
+      <c r="CH21" s="37"/>
+      <c r="CI21" s="37"/>
+      <c r="CJ21" s="37"/>
+      <c r="CK21" s="37"/>
+      <c r="CL21" s="37"/>
+      <c r="CM21" s="37"/>
+      <c r="CN21" s="37"/>
+      <c r="CO21" s="37"/>
+      <c r="CP21" s="37"/>
+      <c r="CQ21" s="37"/>
+      <c r="CR21" s="37"/>
+      <c r="CS21" s="37"/>
+      <c r="CT21" s="37"/>
+      <c r="CU21" s="37"/>
+      <c r="CV21" s="37"/>
+      <c r="CW21" s="37"/>
+      <c r="CX21" s="37"/>
+      <c r="CY21" s="37"/>
+      <c r="CZ21" s="37"/>
+      <c r="DA21" s="37"/>
+      <c r="DB21" s="37"/>
+      <c r="DC21" s="37"/>
+      <c r="DD21" s="37"/>
+      <c r="DE21" s="37"/>
+      <c r="DF21" s="37"/>
+      <c r="DG21" s="37"/>
+      <c r="DH21" s="37"/>
+      <c r="DI21" s="37"/>
+      <c r="DJ21" s="37"/>
+      <c r="DK21" s="37"/>
+      <c r="DL21" s="37"/>
+      <c r="DM21" s="37"/>
+      <c r="DN21" s="37"/>
+      <c r="DO21" s="37"/>
+      <c r="DP21" s="37"/>
+      <c r="DQ21" s="37"/>
+      <c r="DR21" s="37"/>
+      <c r="DS21" s="37"/>
+      <c r="DT21" s="37"/>
+      <c r="DU21" s="37"/>
+      <c r="DV21" s="37"/>
+      <c r="DW21" s="37"/>
+      <c r="DX21" s="37"/>
+      <c r="DY21" s="37"/>
+      <c r="DZ21" s="37"/>
+      <c r="EA21" s="37"/>
+      <c r="EB21" s="37"/>
+      <c r="EC21" s="37"/>
+      <c r="ED21" s="37"/>
+      <c r="EE21" s="37"/>
+      <c r="EF21" s="37"/>
+      <c r="EG21" s="37"/>
+      <c r="EH21" s="37"/>
+      <c r="EI21" s="37"/>
+      <c r="EJ21" s="37"/>
+      <c r="EK21" s="37"/>
+      <c r="EL21" s="37"/>
+      <c r="EM21" s="37"/>
+      <c r="EN21" s="37"/>
+      <c r="EO21" s="37"/>
+      <c r="EP21" s="37"/>
+      <c r="EQ21" s="37"/>
+      <c r="ER21" s="37"/>
+      <c r="ES21" s="37"/>
+      <c r="ET21" s="37"/>
+      <c r="EU21" s="37"/>
+      <c r="EV21" s="37"/>
+      <c r="EW21" s="37"/>
+      <c r="EX21" s="37"/>
+      <c r="EY21" s="37"/>
+      <c r="EZ21" s="37"/>
+      <c r="FA21" s="37"/>
+      <c r="FB21" s="37"/>
+      <c r="FC21" s="37"/>
+      <c r="FD21" s="37"/>
+      <c r="FE21" s="37"/>
+      <c r="FF21" s="37"/>
+      <c r="FG21" s="37"/>
+      <c r="FH21" s="37"/>
+      <c r="FI21" s="37"/>
+      <c r="FJ21" s="37"/>
+      <c r="FK21" s="37"/>
+      <c r="FL21" s="37"/>
+      <c r="FM21" s="37"/>
+      <c r="FN21" s="37"/>
+      <c r="FO21" s="37"/>
+      <c r="FP21" s="37"/>
+      <c r="FQ21" s="37"/>
+      <c r="FR21" s="37"/>
+      <c r="FS21" s="37"/>
+      <c r="FT21" s="37"/>
+      <c r="FU21" s="37"/>
+      <c r="FV21" s="37"/>
+      <c r="FW21" s="37"/>
+      <c r="FX21" s="37"/>
+      <c r="FY21" s="37"/>
+      <c r="FZ21" s="37"/>
+      <c r="GA21" s="37"/>
+      <c r="GB21" s="37"/>
+      <c r="GC21" s="37"/>
+      <c r="GD21" s="37"/>
+      <c r="GE21" s="37"/>
+      <c r="GF21" s="37"/>
+      <c r="GG21" s="37"/>
+      <c r="GH21" s="37"/>
+      <c r="GI21" s="37"/>
+      <c r="GJ21" s="37"/>
+      <c r="GK21" s="37"/>
+      <c r="GL21" s="37"/>
+      <c r="GM21" s="37"/>
+      <c r="GN21" s="37"/>
+      <c r="GO21" s="37"/>
+      <c r="GP21" s="37"/>
+      <c r="GQ21" s="37"/>
+      <c r="GR21" s="37"/>
+      <c r="GS21" s="37"/>
+      <c r="GT21" s="37"/>
+      <c r="GU21" s="37"/>
+      <c r="GV21" s="37"/>
+      <c r="GW21" s="37"/>
+      <c r="GX21" s="37"/>
+      <c r="GY21" s="37"/>
+      <c r="GZ21" s="37"/>
+      <c r="HA21" s="37"/>
+      <c r="HB21" s="37"/>
+      <c r="HC21" s="37"/>
+      <c r="HD21" s="37"/>
+      <c r="HE21" s="37"/>
+      <c r="HF21" s="37"/>
+      <c r="HG21" s="37"/>
+      <c r="HH21" s="37"/>
+      <c r="HI21" s="37"/>
+      <c r="HJ21" s="37"/>
+      <c r="HK21" s="37"/>
+      <c r="HL21" s="37"/>
+      <c r="HM21" s="37"/>
+      <c r="HN21" s="37"/>
+      <c r="HO21" s="37"/>
+      <c r="HP21" s="37"/>
+      <c r="HQ21" s="37"/>
+      <c r="HR21" s="37"/>
+      <c r="HS21" s="37"/>
+      <c r="HT21" s="37"/>
+      <c r="HU21" s="37"/>
+      <c r="HV21" s="37"/>
+      <c r="HW21" s="37"/>
+      <c r="HX21" s="37"/>
+      <c r="HY21" s="37"/>
+      <c r="HZ21" s="37"/>
+      <c r="IA21" s="37"/>
+      <c r="IB21" s="37"/>
+      <c r="IC21" s="37"/>
+      <c r="ID21" s="37"/>
+      <c r="IE21" s="37"/>
+      <c r="IF21" s="37"/>
+      <c r="IG21" s="37"/>
+      <c r="IH21" s="37"/>
+      <c r="II21" s="37"/>
+      <c r="IJ21" s="37"/>
+      <c r="IK21" s="37"/>
+      <c r="IL21" s="37"/>
+      <c r="IM21" s="37"/>
+      <c r="IN21" s="37"/>
+      <c r="IO21" s="37"/>
+      <c r="IP21" s="37"/>
+      <c r="IQ21" s="37"/>
+      <c r="IR21" s="37"/>
+      <c r="IS21" s="37"/>
+      <c r="IT21" s="37"/>
+      <c r="IU21" s="37"/>
+      <c r="IV21" s="37"/>
+      <c r="IW21" s="37"/>
+      <c r="IX21" s="37"/>
+      <c r="IY21" s="37"/>
+      <c r="IZ21" s="37"/>
+      <c r="JA21" s="37"/>
+      <c r="JB21" s="37"/>
+      <c r="JC21" s="37"/>
+      <c r="JD21" s="37"/>
+      <c r="JE21" s="37"/>
+      <c r="JF21" s="37"/>
+      <c r="JG21" s="37"/>
+      <c r="JH21" s="37"/>
+      <c r="JI21" s="37"/>
+      <c r="JJ21" s="37"/>
+      <c r="JK21" s="37"/>
+      <c r="JL21" s="37"/>
+      <c r="JM21" s="37"/>
+      <c r="JN21" s="37"/>
     </row>
     <row r="22" ht="42.75">
-      <c r="A22" s="44" t="s">
-        <v>172</v>
-      </c>
-      <c r="B22" s="44" t="s">
+      <c r="A22" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="B22" s="39" t="s">
         <v>78</v>
       </c>
-      <c r="C22" s="44" t="s">
+      <c r="C22" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="D22" s="44" t="s">
-        <v>173</v>
-      </c>
-      <c r="E22" s="44" t="s">
-        <v>174</v>
-      </c>
-      <c r="F22" s="45" t="s">
+      <c r="D22" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="F22" s="40" t="s">
         <v>107</v>
       </c>
-      <c r="G22" s="44" t="s">
-        <v>175</v>
-      </c>
-      <c r="H22" s="44" t="s">
+      <c r="G22" s="39" t="s">
+        <v>180</v>
+      </c>
+      <c r="H22" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="I22" s="46" t="s">
-        <v>176</v>
-      </c>
-      <c r="J22" s="44" t="s">
-        <v>177</v>
-      </c>
-      <c r="K22" s="47">
+      <c r="I22" s="41" t="s">
+        <v>181</v>
+      </c>
+      <c r="J22" s="39" t="s">
+        <v>182</v>
+      </c>
+      <c r="K22" s="42">
         <v>2010</v>
       </c>
-      <c r="L22" s="47" t="s">
-        <v>178</v>
-      </c>
-      <c r="M22" s="44"/>
-      <c r="N22" s="48" t="s">
-        <v>179</v>
+      <c r="L22" s="42" t="s">
+        <v>183</v>
+      </c>
+      <c r="M22" s="39"/>
+      <c r="N22" s="43" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="23" s="16" customFormat="1" ht="25.5">
-      <c r="A23" s="44" t="s">
-        <v>172</v>
-      </c>
-      <c r="B23" s="44" t="s">
+      <c r="A23" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="B23" s="39" t="s">
         <v>78</v>
       </c>
-      <c r="C23" s="44" t="s">
-        <v>154</v>
-      </c>
-      <c r="D23" s="44" t="s">
-        <v>180</v>
-      </c>
-      <c r="E23" s="47" t="s">
-        <v>181</v>
-      </c>
-      <c r="F23" s="45" t="s">
+      <c r="C23" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="D23" s="39" t="s">
+        <v>185</v>
+      </c>
+      <c r="E23" s="42" t="s">
+        <v>186</v>
+      </c>
+      <c r="F23" s="40" t="s">
         <v>107</v>
       </c>
-      <c r="G23" s="44"/>
-      <c r="H23" s="44" t="s">
+      <c r="G23" s="39"/>
+      <c r="H23" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="I23" s="49" t="s">
-        <v>182</v>
-      </c>
-      <c r="J23" s="44" t="s">
-        <v>139</v>
-      </c>
-      <c r="K23" s="47">
+      <c r="I23" s="44" t="s">
+        <v>187</v>
+      </c>
+      <c r="J23" s="39" t="s">
+        <v>160</v>
+      </c>
+      <c r="K23" s="42">
         <v>2010</v>
       </c>
-      <c r="L23" s="47" t="s">
-        <v>178</v>
-      </c>
-      <c r="M23" s="44"/>
-      <c r="N23" s="50" t="s">
+      <c r="L23" s="42" t="s">
         <v>183</v>
+      </c>
+      <c r="M23" s="39"/>
+      <c r="N23" s="45" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="24" ht="28.5">
-      <c r="A24" s="44" t="s">
-        <v>172</v>
-      </c>
-      <c r="B24" s="44" t="s">
+      <c r="A24" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="39" t="s">
         <v>78</v>
       </c>
-      <c r="C24" s="44" t="s">
-        <v>154</v>
-      </c>
-      <c r="D24" s="44" t="s">
+      <c r="C24" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="D24" s="39" t="s">
+        <v>189</v>
+      </c>
+      <c r="E24" s="39" t="s">
+        <v>189</v>
+      </c>
+      <c r="F24" s="40" t="s">
+        <v>107</v>
+      </c>
+      <c r="G24" s="39"/>
+      <c r="H24" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="I24" s="46" t="s">
+        <v>190</v>
+      </c>
+      <c r="J24" s="39" t="s">
+        <v>160</v>
+      </c>
+      <c r="K24" s="42">
+        <v>2010</v>
+      </c>
+      <c r="L24" s="42" t="s">
+        <v>183</v>
+      </c>
+      <c r="M24" s="39"/>
+      <c r="N24" s="43" t="s">
         <v>184</v>
-      </c>
-      <c r="E24" s="44" t="s">
-        <v>184</v>
-      </c>
-      <c r="F24" s="45" t="s">
-        <v>107</v>
-      </c>
-      <c r="G24" s="44"/>
-      <c r="H24" s="44" t="s">
-        <v>21</v>
-      </c>
-      <c r="I24" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="J24" s="44" t="s">
-        <v>139</v>
-      </c>
-      <c r="K24" s="47">
-        <v>2010</v>
-      </c>
-      <c r="L24" s="47" t="s">
-        <v>178</v>
-      </c>
-      <c r="M24" s="44"/>
-      <c r="N24" s="48" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="25" ht="25.5">
-      <c r="A25" s="52" t="s">
-        <v>186</v>
-      </c>
-      <c r="B25" s="52" t="s">
+      <c r="A25" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="B25" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="52" t="s">
-        <v>187</v>
-      </c>
-      <c r="D25" s="52" t="s">
-        <v>188</v>
-      </c>
-      <c r="E25" s="52" t="s">
-        <v>189</v>
-      </c>
-      <c r="F25" s="53" t="s">
-        <v>190</v>
-      </c>
-      <c r="G25" s="52"/>
-      <c r="H25" s="52"/>
-      <c r="I25" s="54" t="s">
-        <v>191</v>
-      </c>
-      <c r="J25" s="52"/>
-      <c r="K25" s="52">
+      <c r="C25" s="47" t="s">
+        <v>192</v>
+      </c>
+      <c r="D25" s="47" t="s">
+        <v>193</v>
+      </c>
+      <c r="E25" s="47" t="s">
+        <v>194</v>
+      </c>
+      <c r="F25" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="G25" s="47"/>
+      <c r="H25" s="47"/>
+      <c r="I25" s="49" t="s">
+        <v>196</v>
+      </c>
+      <c r="J25" s="47"/>
+      <c r="K25" s="47">
         <v>2016</v>
       </c>
-      <c r="L25" s="52" t="s">
-        <v>192</v>
-      </c>
-      <c r="M25" s="52"/>
+      <c r="L25" s="47" t="s">
+        <v>197</v>
+      </c>
+      <c r="M25" s="47"/>
       <c r="N25" s="25"/>
     </row>
     <row r="26" ht="25.5">
-      <c r="A26" s="52" t="s">
-        <v>186</v>
-      </c>
-      <c r="B26" s="52" t="s">
+      <c r="A26" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="B26" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="C26" s="52" t="s">
-        <v>187</v>
-      </c>
-      <c r="D26" s="52" t="s">
-        <v>193</v>
-      </c>
-      <c r="E26" s="52" t="s">
-        <v>189</v>
-      </c>
-      <c r="F26" s="53" t="s">
+      <c r="C26" s="47" t="s">
+        <v>192</v>
+      </c>
+      <c r="D26" s="47" t="s">
+        <v>198</v>
+      </c>
+      <c r="E26" s="47" t="s">
         <v>194</v>
       </c>
-      <c r="G26" s="52"/>
-      <c r="H26" s="52"/>
-      <c r="I26" s="55"/>
-      <c r="J26" s="56"/>
-      <c r="K26" s="52"/>
-      <c r="L26" s="52"/>
-      <c r="M26" s="52"/>
+      <c r="F26" s="48" t="s">
+        <v>199</v>
+      </c>
+      <c r="G26" s="47"/>
+      <c r="H26" s="47"/>
+      <c r="I26" s="50"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="47"/>
+      <c r="L26" s="47"/>
+      <c r="M26" s="47"/>
       <c r="N26" s="25"/>
     </row>
     <row r="27" ht="25.5">
-      <c r="A27" s="52" t="s">
-        <v>186</v>
-      </c>
-      <c r="B27" s="52" t="s">
+      <c r="A27" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="B27" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="C27" s="52" t="s">
-        <v>195</v>
-      </c>
-      <c r="D27" s="52" t="s">
-        <v>196</v>
-      </c>
-      <c r="E27" s="52" t="s">
-        <v>197</v>
-      </c>
-      <c r="F27" s="52" t="s">
-        <v>198</v>
-      </c>
-      <c r="G27" s="52"/>
-      <c r="H27" s="52"/>
-      <c r="I27" s="54" t="s">
-        <v>199</v>
-      </c>
-      <c r="J27" s="57"/>
-      <c r="K27" s="52"/>
-      <c r="L27" s="52"/>
-      <c r="M27" s="52"/>
+      <c r="C27" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="D27" s="47" t="s">
+        <v>201</v>
+      </c>
+      <c r="E27" s="47" t="s">
+        <v>202</v>
+      </c>
+      <c r="F27" s="47" t="s">
+        <v>203</v>
+      </c>
+      <c r="G27" s="47"/>
+      <c r="H27" s="47"/>
+      <c r="I27" s="49" t="s">
+        <v>204</v>
+      </c>
+      <c r="J27" s="52"/>
+      <c r="K27" s="47"/>
+      <c r="L27" s="47"/>
+      <c r="M27" s="47"/>
       <c r="N27" s="25"/>
     </row>
     <row r="28" ht="38.25">
-      <c r="A28" s="52" t="s">
-        <v>186</v>
-      </c>
-      <c r="B28" s="52" t="s">
+      <c r="A28" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="B28" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="52" t="s">
+      <c r="C28" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="52" t="s">
-        <v>200</v>
-      </c>
-      <c r="E28" s="52" t="s">
-        <v>201</v>
-      </c>
-      <c r="F28" s="58" t="s">
-        <v>202</v>
-      </c>
-      <c r="G28" s="52" t="s">
-        <v>203</v>
-      </c>
-      <c r="H28" s="52" t="s">
+      <c r="D28" s="47" t="s">
+        <v>205</v>
+      </c>
+      <c r="E28" s="47" t="s">
+        <v>206</v>
+      </c>
+      <c r="F28" s="53" t="s">
+        <v>207</v>
+      </c>
+      <c r="G28" s="47" t="s">
+        <v>208</v>
+      </c>
+      <c r="H28" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="I28" s="59" t="s">
-        <v>204</v>
-      </c>
-      <c r="J28" s="52" t="s">
-        <v>205</v>
-      </c>
-      <c r="K28" s="52"/>
-      <c r="L28" s="52" t="s">
+      <c r="I28" s="54" t="s">
+        <v>209</v>
+      </c>
+      <c r="J28" s="47" t="s">
+        <v>210</v>
+      </c>
+      <c r="K28" s="47"/>
+      <c r="L28" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="M28" s="52"/>
-      <c r="N28" s="60" t="s">
-        <v>206</v>
+      <c r="M28" s="47"/>
+      <c r="N28" s="55" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="29" ht="89.25">
-      <c r="A29" s="52" t="s">
-        <v>186</v>
-      </c>
-      <c r="B29" s="52" t="s">
+      <c r="A29" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="B29" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="52" t="s">
+      <c r="C29" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="D29" s="52" t="s">
-        <v>207</v>
-      </c>
-      <c r="E29" s="52" t="s">
-        <v>208</v>
-      </c>
-      <c r="F29" s="52" t="s">
+      <c r="D29" s="47" t="s">
+        <v>212</v>
+      </c>
+      <c r="E29" s="47" t="s">
+        <v>213</v>
+      </c>
+      <c r="F29" s="47" t="s">
         <v>82</v>
       </c>
-      <c r="G29" s="52" t="s">
-        <v>209</v>
-      </c>
-      <c r="H29" s="52" t="s">
+      <c r="G29" s="47" t="s">
+        <v>214</v>
+      </c>
+      <c r="H29" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="I29" s="59" t="s">
+      <c r="I29" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="J29" s="52" t="s">
-        <v>210</v>
-      </c>
-      <c r="K29" s="52" t="s">
+      <c r="J29" s="47" t="s">
+        <v>215</v>
+      </c>
+      <c r="K29" s="47" t="s">
         <v>93</v>
       </c>
-      <c r="L29" s="52" t="s">
+      <c r="L29" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="M29" s="52"/>
-      <c r="N29" s="60" t="s">
-        <v>206</v>
+      <c r="M29" s="47"/>
+      <c r="N29" s="55" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="30" ht="25.5">
-      <c r="A30" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B30" s="61" t="s">
+      <c r="A30" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B30" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="C30" s="61" t="s">
+      <c r="C30" s="56" t="s">
         <v>79</v>
       </c>
-      <c r="D30" s="61" t="s">
-        <v>212</v>
-      </c>
-      <c r="E30" s="61" t="s">
-        <v>213</v>
-      </c>
-      <c r="F30" s="62"/>
-      <c r="G30" s="61"/>
-      <c r="H30" s="61"/>
-      <c r="I30" s="63" t="s">
-        <v>214</v>
-      </c>
-      <c r="J30" s="64"/>
-      <c r="K30" s="61"/>
-      <c r="L30" s="61" t="s">
-        <v>215</v>
-      </c>
-      <c r="M30" s="61"/>
-      <c r="N30" s="36"/>
+      <c r="D30" s="56" t="s">
+        <v>217</v>
+      </c>
+      <c r="E30" s="56" t="s">
+        <v>218</v>
+      </c>
+      <c r="F30" s="57"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="56"/>
+      <c r="I30" s="58" t="s">
+        <v>219</v>
+      </c>
+      <c r="J30" s="59"/>
+      <c r="K30" s="56"/>
+      <c r="L30" s="56" t="s">
+        <v>220</v>
+      </c>
+      <c r="M30" s="56"/>
+      <c r="N30" s="60"/>
     </row>
     <row r="31" ht="25.5">
-      <c r="A31" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B31" s="61" t="s">
+      <c r="A31" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B31" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="C31" s="61" t="s">
+      <c r="C31" s="56" t="s">
         <v>79</v>
       </c>
-      <c r="D31" s="61" t="s">
-        <v>216</v>
-      </c>
-      <c r="E31" s="61" t="s">
-        <v>213</v>
-      </c>
-      <c r="F31" s="62"/>
-      <c r="G31" s="61"/>
-      <c r="H31" s="61"/>
-      <c r="I31" s="63" t="s">
-        <v>217</v>
-      </c>
-      <c r="J31" s="61"/>
-      <c r="K31" s="61"/>
-      <c r="L31" s="61"/>
-      <c r="M31" s="61"/>
-      <c r="N31" s="36"/>
+      <c r="D31" s="56" t="s">
+        <v>221</v>
+      </c>
+      <c r="E31" s="56" t="s">
+        <v>218</v>
+      </c>
+      <c r="F31" s="57"/>
+      <c r="G31" s="56"/>
+      <c r="H31" s="56"/>
+      <c r="I31" s="58" t="s">
+        <v>222</v>
+      </c>
+      <c r="J31" s="56"/>
+      <c r="K31" s="56"/>
+      <c r="L31" s="56"/>
+      <c r="M31" s="56"/>
+      <c r="N31" s="60"/>
     </row>
     <row r="32" ht="25.5">
-      <c r="A32" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B32" s="61" t="s">
+      <c r="A32" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B32" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="C32" s="61" t="s">
+      <c r="C32" s="56" t="s">
         <v>79</v>
       </c>
-      <c r="D32" s="61" t="s">
+      <c r="D32" s="56" t="s">
+        <v>223</v>
+      </c>
+      <c r="E32" s="56" t="s">
         <v>218</v>
       </c>
-      <c r="E32" s="61" t="s">
-        <v>213</v>
-      </c>
-      <c r="F32" s="62"/>
-      <c r="G32" s="61"/>
-      <c r="H32" s="61"/>
-      <c r="I32" s="63" t="s">
-        <v>214</v>
-      </c>
-      <c r="J32" s="64"/>
-      <c r="K32" s="61"/>
-      <c r="L32" s="61" t="s">
-        <v>215</v>
-      </c>
-      <c r="M32" s="61"/>
-      <c r="N32" s="36"/>
+      <c r="F32" s="57"/>
+      <c r="G32" s="56"/>
+      <c r="H32" s="56"/>
+      <c r="I32" s="58" t="s">
+        <v>219</v>
+      </c>
+      <c r="J32" s="59"/>
+      <c r="K32" s="56"/>
+      <c r="L32" s="56" t="s">
+        <v>220</v>
+      </c>
+      <c r="M32" s="56"/>
+      <c r="N32" s="60"/>
     </row>
     <row r="33" ht="25.5">
-      <c r="A33" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B33" s="61" t="s">
+      <c r="A33" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B33" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="61" t="s">
-        <v>154</v>
-      </c>
-      <c r="D33" s="61" t="s">
-        <v>219</v>
-      </c>
-      <c r="E33" s="61"/>
-      <c r="F33" s="62" t="s">
-        <v>220</v>
-      </c>
-      <c r="G33" s="61"/>
-      <c r="H33" s="61"/>
-      <c r="I33" s="65"/>
-      <c r="J33" s="61"/>
-      <c r="K33" s="61"/>
-      <c r="L33" s="61"/>
-      <c r="M33" s="61"/>
-      <c r="N33" s="36"/>
+      <c r="C33" s="56" t="s">
+        <v>128</v>
+      </c>
+      <c r="D33" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="E33" s="56"/>
+      <c r="F33" s="57" t="s">
+        <v>225</v>
+      </c>
+      <c r="G33" s="56"/>
+      <c r="H33" s="56"/>
+      <c r="I33" s="61"/>
+      <c r="J33" s="56"/>
+      <c r="K33" s="56"/>
+      <c r="L33" s="56"/>
+      <c r="M33" s="56"/>
+      <c r="N33" s="60"/>
     </row>
     <row r="34" ht="25.5">
-      <c r="A34" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B34" s="61" t="s">
+      <c r="A34" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B34" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="C34" s="61" t="s">
-        <v>195</v>
-      </c>
-      <c r="D34" s="61" t="s">
-        <v>221</v>
-      </c>
-      <c r="E34" s="61" t="s">
-        <v>213</v>
-      </c>
-      <c r="F34" s="62"/>
-      <c r="G34" s="61"/>
-      <c r="H34" s="61"/>
-      <c r="I34" s="66"/>
-      <c r="J34" s="61"/>
-      <c r="K34" s="61"/>
-      <c r="L34" s="61"/>
-      <c r="M34" s="61"/>
-      <c r="N34" s="36"/>
+      <c r="C34" s="56" t="s">
+        <v>200</v>
+      </c>
+      <c r="D34" s="56" t="s">
+        <v>226</v>
+      </c>
+      <c r="E34" s="56" t="s">
+        <v>218</v>
+      </c>
+      <c r="F34" s="57"/>
+      <c r="G34" s="56"/>
+      <c r="H34" s="56"/>
+      <c r="I34" s="62"/>
+      <c r="J34" s="56"/>
+      <c r="K34" s="56"/>
+      <c r="L34" s="56"/>
+      <c r="M34" s="56"/>
+      <c r="N34" s="60"/>
     </row>
     <row r="35" ht="38.25">
-      <c r="A35" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B35" s="61" t="s">
+      <c r="A35" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B35" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="C35" s="61" t="s">
-        <v>195</v>
-      </c>
-      <c r="D35" s="61" t="s">
-        <v>222</v>
-      </c>
-      <c r="E35" s="61" t="s">
-        <v>213</v>
-      </c>
-      <c r="F35" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="G35" s="61"/>
-      <c r="H35" s="61"/>
-      <c r="I35" s="63" t="s">
-        <v>224</v>
-      </c>
-      <c r="J35" s="61"/>
-      <c r="K35" s="61"/>
-      <c r="L35" s="61"/>
-      <c r="M35" s="61"/>
-      <c r="N35" s="36"/>
+      <c r="C35" s="56" t="s">
+        <v>200</v>
+      </c>
+      <c r="D35" s="56" t="s">
+        <v>227</v>
+      </c>
+      <c r="E35" s="56" t="s">
+        <v>218</v>
+      </c>
+      <c r="F35" s="57" t="s">
+        <v>228</v>
+      </c>
+      <c r="G35" s="56"/>
+      <c r="H35" s="56"/>
+      <c r="I35" s="58" t="s">
+        <v>229</v>
+      </c>
+      <c r="J35" s="56"/>
+      <c r="K35" s="56"/>
+      <c r="L35" s="56"/>
+      <c r="M35" s="56"/>
+      <c r="N35" s="60"/>
     </row>
     <row r="36" ht="38.25">
-      <c r="A36" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B36" s="61" t="s">
+      <c r="A36" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B36" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="C36" s="61" t="s">
-        <v>225</v>
-      </c>
-      <c r="D36" s="61" t="s">
-        <v>226</v>
-      </c>
-      <c r="E36" s="61" t="s">
-        <v>227</v>
-      </c>
-      <c r="F36" s="62" t="s">
-        <v>228</v>
-      </c>
-      <c r="G36" s="61"/>
-      <c r="H36" s="61"/>
-      <c r="I36" s="63" t="s">
-        <v>229</v>
-      </c>
-      <c r="J36" s="61"/>
-      <c r="K36" s="61"/>
-      <c r="L36" s="61" t="s">
+      <c r="C36" s="56" t="s">
+        <v>230</v>
+      </c>
+      <c r="D36" s="56" t="s">
+        <v>231</v>
+      </c>
+      <c r="E36" s="56" t="s">
+        <v>232</v>
+      </c>
+      <c r="F36" s="57" t="s">
+        <v>233</v>
+      </c>
+      <c r="G36" s="56"/>
+      <c r="H36" s="56"/>
+      <c r="I36" s="58" t="s">
+        <v>234</v>
+      </c>
+      <c r="J36" s="56"/>
+      <c r="K36" s="56"/>
+      <c r="L36" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="M36" s="61"/>
-      <c r="N36" s="36"/>
+      <c r="M36" s="56"/>
+      <c r="N36" s="60"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B37" s="61" t="s">
+      <c r="A37" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B37" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="61" t="s">
-        <v>230</v>
-      </c>
-      <c r="D37" s="61" t="s">
-        <v>231</v>
-      </c>
-      <c r="E37" s="61" t="s">
-        <v>213</v>
-      </c>
-      <c r="F37" s="61"/>
-      <c r="G37" s="61"/>
-      <c r="H37" s="61"/>
-      <c r="I37" s="67"/>
-      <c r="J37" s="61"/>
-      <c r="K37" s="61"/>
-      <c r="L37" s="61"/>
-      <c r="M37" s="61"/>
-      <c r="N37" s="61" t="s">
-        <v>232</v>
+      <c r="C37" s="56" t="s">
+        <v>235</v>
+      </c>
+      <c r="D37" s="56" t="s">
+        <v>236</v>
+      </c>
+      <c r="E37" s="56" t="s">
+        <v>218</v>
+      </c>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="63"/>
+      <c r="J37" s="56"/>
+      <c r="K37" s="56"/>
+      <c r="L37" s="56"/>
+      <c r="M37" s="56"/>
+      <c r="N37" s="56" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="38" ht="51">
-      <c r="A38" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B38" s="61" t="s">
+      <c r="A38" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B38" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="61" t="s">
-        <v>230</v>
-      </c>
-      <c r="D38" s="61" t="s">
-        <v>233</v>
-      </c>
-      <c r="E38" s="61" t="s">
-        <v>213</v>
-      </c>
-      <c r="F38" s="61"/>
-      <c r="G38" s="61"/>
-      <c r="H38" s="61"/>
-      <c r="I38" s="67"/>
-      <c r="J38" s="61"/>
-      <c r="K38" s="61"/>
-      <c r="L38" s="61"/>
-      <c r="M38" s="61"/>
-      <c r="N38" s="61" t="s">
-        <v>232</v>
+      <c r="C38" s="56" t="s">
+        <v>235</v>
+      </c>
+      <c r="D38" s="56" t="s">
+        <v>238</v>
+      </c>
+      <c r="E38" s="56" t="s">
+        <v>218</v>
+      </c>
+      <c r="F38" s="56"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="56"/>
+      <c r="I38" s="63"/>
+      <c r="J38" s="56"/>
+      <c r="K38" s="56"/>
+      <c r="L38" s="56"/>
+      <c r="M38" s="56"/>
+      <c r="N38" s="56" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="39" ht="51">
-      <c r="A39" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B39" s="61" t="s">
+      <c r="A39" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B39" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C39" s="61" t="s">
-        <v>234</v>
-      </c>
-      <c r="D39" s="61" t="s">
-        <v>235</v>
-      </c>
-      <c r="E39" s="61" t="s">
-        <v>236</v>
-      </c>
-      <c r="F39" s="68" t="s">
+      <c r="C39" s="56" t="s">
+        <v>239</v>
+      </c>
+      <c r="D39" s="56" t="s">
+        <v>240</v>
+      </c>
+      <c r="E39" s="56" t="s">
+        <v>241</v>
+      </c>
+      <c r="F39" s="64" t="s">
+        <v>242</v>
+      </c>
+      <c r="G39" s="56"/>
+      <c r="H39" s="56"/>
+      <c r="I39" s="63"/>
+      <c r="J39" s="56"/>
+      <c r="K39" s="56"/>
+      <c r="L39" s="56"/>
+      <c r="M39" s="56"/>
+      <c r="N39" s="56" t="s">
         <v>237</v>
-      </c>
-      <c r="G39" s="61"/>
-      <c r="H39" s="61"/>
-      <c r="I39" s="67"/>
-      <c r="J39" s="61"/>
-      <c r="K39" s="61"/>
-      <c r="L39" s="61"/>
-      <c r="M39" s="61"/>
-      <c r="N39" s="61" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="40" s="10" customFormat="1" ht="25.5">
-      <c r="A40" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="B40" s="61" t="s">
+      <c r="A40" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B40" s="56" t="s">
         <v>36</v>
       </c>
-      <c r="C40" s="61" t="s">
+      <c r="C40" s="56" t="s">
         <v>68</v>
       </c>
-      <c r="D40" s="61" t="s">
-        <v>238</v>
-      </c>
-      <c r="E40" s="61" t="s">
-        <v>213</v>
-      </c>
-      <c r="F40" s="61"/>
-      <c r="G40" s="61"/>
-      <c r="H40" s="61"/>
-      <c r="I40" s="67"/>
-      <c r="J40" s="61"/>
-      <c r="K40" s="61"/>
-      <c r="L40" s="61"/>
-      <c r="M40" s="61"/>
-      <c r="N40" s="61" t="s">
-        <v>232</v>
+      <c r="D40" s="56" t="s">
+        <v>243</v>
+      </c>
+      <c r="E40" s="56" t="s">
+        <v>218</v>
+      </c>
+      <c r="F40" s="56"/>
+      <c r="G40" s="56"/>
+      <c r="H40" s="56"/>
+      <c r="I40" s="63"/>
+      <c r="J40" s="56"/>
+      <c r="K40" s="56"/>
+      <c r="L40" s="56"/>
+      <c r="M40" s="56"/>
+      <c r="N40" s="56" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="41" ht="14.25">
-      <c r="A41" s="69" t="s">
-        <v>239</v>
-      </c>
-      <c r="B41" s="69" t="s">
+      <c r="A41" s="65" t="s">
+        <v>244</v>
+      </c>
+      <c r="B41" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C41" s="69" t="s">
+      <c r="C41" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="D41" s="69" t="s">
-        <v>240</v>
-      </c>
-      <c r="E41" s="69" t="s">
-        <v>241</v>
-      </c>
-      <c r="F41" s="69"/>
-      <c r="G41" s="69" t="s">
-        <v>242</v>
-      </c>
-      <c r="H41" s="69" t="s">
+      <c r="D41" s="65" t="s">
+        <v>245</v>
+      </c>
+      <c r="E41" s="65" t="s">
+        <v>246</v>
+      </c>
+      <c r="F41" s="65"/>
+      <c r="G41" s="65" t="s">
+        <v>247</v>
+      </c>
+      <c r="H41" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="I41" s="70"/>
-      <c r="J41" s="69"/>
-      <c r="K41" s="69"/>
-      <c r="L41" s="69"/>
-      <c r="M41" s="69" t="s">
-        <v>140</v>
-      </c>
-      <c r="N41" s="69"/>
+      <c r="I41" s="66"/>
+      <c r="J41" s="65"/>
+      <c r="K41" s="65"/>
+      <c r="L41" s="65"/>
+      <c r="M41" s="65" t="s">
+        <v>161</v>
+      </c>
+      <c r="N41" s="65"/>
     </row>
     <row r="42" ht="14.25">
       <c r="A42" s="1"/>
-      <c r="M42" s="71"/>
-      <c r="N42" s="71"/>
+      <c r="M42" s="67"/>
+      <c r="N42" s="67"/>
     </row>
     <row r="43" ht="14.25">
-      <c r="M43" s="71"/>
-      <c r="N43" s="71"/>
+      <c r="M43" s="67"/>
+      <c r="N43" s="67"/>
     </row>
     <row r="44" ht="14.25">
-      <c r="M44" s="71"/>
-      <c r="N44" s="71"/>
+      <c r="M44" s="67"/>
+      <c r="N44" s="67"/>
     </row>
     <row r="45" ht="14.25">
-      <c r="M45" s="71"/>
-      <c r="N45" s="71"/>
+      <c r="M45" s="67"/>
+      <c r="N45" s="67"/>
     </row>
     <row r="46" ht="14.25">
-      <c r="M46" s="71"/>
-      <c r="N46" s="71"/>
+      <c r="M46" s="67"/>
+      <c r="N46" s="67"/>
     </row>
     <row r="47" ht="14.25">
-      <c r="M47" s="71"/>
-      <c r="N47" s="71"/>
+      <c r="M47" s="67"/>
+      <c r="N47" s="67"/>
     </row>
     <row r="48" ht="14.25">
-      <c r="M48" s="71"/>
-      <c r="N48" s="71"/>
+      <c r="M48" s="67"/>
+      <c r="N48" s="67"/>
     </row>
     <row r="49" ht="14.25">
-      <c r="M49" s="71"/>
-      <c r="N49" s="71"/>
+      <c r="M49" s="67"/>
+      <c r="N49" s="67"/>
     </row>
     <row r="50" ht="14.25">
-      <c r="M50" s="71"/>
-      <c r="N50" s="71"/>
+      <c r="M50" s="67"/>
+      <c r="N50" s="67"/>
     </row>
     <row r="51" ht="14.25">
-      <c r="M51" s="71"/>
-      <c r="N51" s="71"/>
+      <c r="M51" s="67"/>
+      <c r="N51" s="67"/>
     </row>
     <row r="52" ht="14.25">
-      <c r="M52" s="71"/>
-      <c r="N52" s="71"/>
+      <c r="M52" s="67"/>
+      <c r="N52" s="67"/>
     </row>
     <row r="53" ht="14.25">
-      <c r="M53" s="71"/>
-      <c r="N53" s="71"/>
+      <c r="M53" s="67"/>
+      <c r="N53" s="67"/>
     </row>
     <row r="54" ht="14.25">
-      <c r="M54" s="71"/>
-      <c r="N54" s="71"/>
+      <c r="M54" s="67"/>
+      <c r="N54" s="67"/>
     </row>
     <row r="55" ht="14.25">
-      <c r="M55" s="71"/>
-      <c r="N55" s="71"/>
+      <c r="M55" s="67"/>
+      <c r="N55" s="67"/>
     </row>
     <row r="56" ht="14.25">
-      <c r="M56" s="71"/>
-      <c r="N56" s="71"/>
+      <c r="M56" s="67"/>
+      <c r="N56" s="67"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N41">
@@ -8615,9 +8645,9 @@
     <hyperlink r:id="rId9" ref="I13"/>
     <hyperlink r:id="rId10" location="c=indicator&amp;i=stru_2020_1.pbs20&amp;t=A02&amp;view=map11" ref="I14"/>
     <hyperlink r:id="rId11" ref="I15"/>
-    <hyperlink r:id="rId12" ref="I17"/>
-    <hyperlink r:id="rId13" ref="I18"/>
-    <hyperlink r:id="rId14" ref="I19"/>
+    <hyperlink r:id="rId12" ref="I16"/>
+    <hyperlink r:id="rId13" ref="I17"/>
+    <hyperlink r:id="rId14" ref="I18"/>
     <hyperlink r:id="rId15" ref="I20"/>
     <hyperlink r:id="rId16" ref="I21"/>
     <hyperlink r:id="rId17" ref="I22"/>
@@ -8649,60 +8679,60 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
-      <c r="A1" s="72" t="s">
-        <v>243</v>
-      </c>
-      <c r="B1" s="72" t="s">
-        <v>244</v>
+      <c r="A1" s="68" t="s">
+        <v>248</v>
+      </c>
+      <c r="B1" s="68" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="2" s="0" customFormat="1" ht="14.25">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="74" t="s">
-        <v>245</v>
+      <c r="B2" s="70" t="s">
+        <v>250</v>
       </c>
       <c r="C2"/>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="27" t="s">
-        <v>132</v>
+      <c r="A3" s="29" t="s">
+        <v>153</v>
       </c>
       <c r="B3" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="44" t="s">
-        <v>172</v>
+      <c r="A4" s="39" t="s">
+        <v>177</v>
       </c>
       <c r="B4" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="52" t="s">
-        <v>186</v>
+      <c r="A5" s="47" t="s">
+        <v>191</v>
       </c>
       <c r="B5" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="61" t="s">
-        <v>211</v>
+      <c r="A6" s="56" t="s">
+        <v>216</v>
       </c>
       <c r="B6" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="69" t="s">
-        <v>239</v>
+      <c r="A7" s="65" t="s">
+        <v>244</v>
       </c>
       <c r="B7" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -8725,20 +8755,20 @@
     <col customWidth="1" min="6" max="6" width="12.8515625"/>
     <col bestFit="1" customWidth="1" min="7" max="7" width="25.78125"/>
     <col bestFit="1" customWidth="1" min="8" max="8" width="21.3515625"/>
-    <col customWidth="1" min="9" max="9" style="75" width="32.7109375"/>
+    <col customWidth="1" min="9" max="9" style="71" width="32.7109375"/>
     <col customWidth="1" min="10" max="10" width="23.57421875"/>
     <col customWidth="1" min="11" max="11" width="44.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" s="72" customFormat="1" ht="25.5">
-      <c r="A1" s="72" t="s">
+    <row r="1" s="68" customFormat="1" ht="25.5">
+      <c r="A1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="72" t="s">
-        <v>251</v>
-      </c>
-      <c r="C1" s="72" t="s">
-        <v>252</v>
+      <c r="B1" s="68" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1" s="68" t="s">
+        <v>257</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>9</v>
@@ -8755,49 +8785,49 @@
       <c r="H1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="76" t="s">
-        <v>253</v>
-      </c>
-      <c r="J1" s="72" t="s">
-        <v>254</v>
-      </c>
-      <c r="K1" s="72" t="s">
+      <c r="I1" s="72" t="s">
+        <v>258</v>
+      </c>
+      <c r="J1" s="68" t="s">
+        <v>259</v>
+      </c>
+      <c r="K1" s="68" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" s="77" customFormat="1" ht="28.5">
-      <c r="A2" s="78" t="s">
+    <row r="2" s="73" customFormat="1" ht="28.5">
+      <c r="A2" s="74" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="79" t="s">
-        <v>255</v>
-      </c>
-      <c r="C2" s="78" t="s">
-        <v>256</v>
-      </c>
-      <c r="D2" s="79" t="s">
-        <v>257</v>
-      </c>
-      <c r="E2" s="79" t="s">
-        <v>258</v>
-      </c>
-      <c r="F2" s="79" t="s">
-        <v>259</v>
-      </c>
-      <c r="G2" s="77" t="s">
+      <c r="B2" s="75" t="s">
         <v>260</v>
       </c>
-      <c r="H2" s="78" t="s">
+      <c r="C2" s="74" t="s">
         <v>261</v>
       </c>
-      <c r="I2" s="80" t="s">
+      <c r="D2" s="75" t="s">
         <v>262</v>
       </c>
-      <c r="J2" s="77" t="s">
+      <c r="E2" s="75" t="s">
         <v>263</v>
       </c>
-      <c r="K2" s="81" t="s">
+      <c r="F2" s="75" t="s">
         <v>264</v>
+      </c>
+      <c r="G2" s="73" t="s">
+        <v>265</v>
+      </c>
+      <c r="H2" s="74" t="s">
+        <v>266</v>
+      </c>
+      <c r="I2" s="76" t="s">
+        <v>267</v>
+      </c>
+      <c r="J2" s="73" t="s">
+        <v>268</v>
+      </c>
+      <c r="K2" s="77" t="s">
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>